<commit_message>
feat: add ZIP upload support and enhance auth UI
- Enable ZIP file uploads for DIAN XML processing.
- Improve feedback messages for batch uploads.
- Implement restricted navigation logic in AuthModal for non-admin users.
- Add global custom scrollbar styling.
</commit_message>
<xml_diff>
--- a/data/tlm_base_de_datos_maestra.xlsx
+++ b/data/tlm_base_de_datos_maestra.xlsx
@@ -433,7 +433,7 @@
         <v>Fecha de Generación</v>
       </c>
       <c r="B3" t="str">
-        <v>14/10/2026, 3:26:43 p. m.</v>
+        <v>22/10/2026, 10:50:53 a. m.</v>
       </c>
     </row>
     <row r="4">
@@ -457,7 +457,7 @@
         <v>Empresa Principal</v>
       </c>
       <c r="B6" t="str">
-        <v>TLM Consulting S.A.S. (Principal)</v>
+        <v>TLM Automatizaciones y Consultoría S.A.S.</v>
       </c>
     </row>
     <row r="7">
@@ -465,7 +465,7 @@
         <v>NIT Principal</v>
       </c>
       <c r="B7" t="str">
-        <v>901234567-8</v>
+        <v>901.458.789-2</v>
       </c>
     </row>
     <row r="8">
@@ -473,7 +473,7 @@
         <v>Total Facturas DIAN Registradas</v>
       </c>
       <c r="B8">
-        <v>6</v>
+        <v>8</v>
       </c>
     </row>
     <row r="9">
@@ -489,7 +489,7 @@
         <v>Total Terceros en Balance</v>
       </c>
       <c r="B10">
-        <v>3</v>
+        <v>6</v>
       </c>
     </row>
     <row r="11">
@@ -537,7 +537,7 @@
         <v>Auditorías &amp; Commits Registrados</v>
       </c>
       <c r="B16">
-        <v>12</v>
+        <v>16</v>
       </c>
     </row>
     <row r="17">
@@ -545,7 +545,7 @@
         <v>Valor Total Compras Facturadas (COP)</v>
       </c>
       <c r="B17" t="str">
-        <v>$24.920.100</v>
+        <v>$35.653.567</v>
       </c>
     </row>
     <row r="18">
@@ -565,7 +565,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:K13"/>
+  <dimension ref="A1:K17"/>
   <cols>
     <col min="1" max="1" width="14.83203125" customWidth="1"/>
     <col min="2" max="2" width="24.83203125" customWidth="1"/>
@@ -617,28 +617,22 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>mod-1792009185879-522</v>
+        <v>mod-sql-otaz37l</v>
       </c>
       <c r="B2" t="str">
-        <v>2026-10-14T20:19:45.879Z</v>
+        <v>2026-10-22 14:10:11.838+00</v>
       </c>
       <c r="C2" t="str">
-        <v>Juan Yaya - Administrador Maestro</v>
-      </c>
-      <c r="D2" t="str">
-        <v>automatizaciones@tlm.net.co</v>
-      </c>
-      <c r="E2" t="str">
-        <v>Administrador</v>
+        <v>Juan Yaya</v>
       </c>
       <c r="F2" t="str">
-        <v>GCP_SYNC</v>
+        <v>FACTURA_UPDATE</v>
       </c>
       <c r="G2" t="str">
-        <v>Sincronización y despliegue del Repositorio v2.0 a Google Cloud Platform (gcp-a5e57g3)</v>
+        <v>Ajuste tributario F350 en SMVP137803: tarifa 4%, casilla 62</v>
       </c>
       <c r="H2" t="str">
-        <v>v2-7d9f1bb</v>
+        <v>csql-2b21t39</v>
       </c>
       <c r="I2" t="str">
         <v>v2.0</v>
@@ -647,33 +641,27 @@
         <v>Repositorio Central de Juan Yaya</v>
       </c>
       <c r="K2" t="str">
-        <v>Sincronización instantánea del Repositorio v2.0 a Google Cloud Platform (us-east1).</v>
+        <v>Retención calculada en Cloud SQL: $60.852 COP.</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>mod-1792008839125-868</v>
+        <v>mod-sql-j6np45l</v>
       </c>
       <c r="B3" t="str">
-        <v>2026-10-14T20:13:59.125Z</v>
+        <v>2026-10-22 14:10:10.434+00</v>
       </c>
       <c r="C3" t="str">
         <v>Juan Yaya</v>
       </c>
-      <c r="D3" t="str">
-        <v>automatizaciones@tlm.net.co</v>
-      </c>
-      <c r="E3" t="str">
-        <v>Administrador</v>
-      </c>
       <c r="F3" t="str">
-        <v>GCP_SYNC</v>
+        <v>FACTURA_UPDATE</v>
       </c>
       <c r="G3" t="str">
-        <v>Sincronización de 7 identidades con Google Cloud IAM (iam-760rd55)</v>
+        <v>Ajuste tributario F350 en SMVP137803: tarifa 10%, casilla 61</v>
       </c>
       <c r="H3" t="str">
-        <v>v2-2af7b79</v>
+        <v>csql-mrh3o41</v>
       </c>
       <c r="I3" t="str">
         <v>v2.0</v>
@@ -682,33 +670,27 @@
         <v>Repositorio Central de Juan Yaya</v>
       </c>
       <c r="K3" t="str">
-        <v>Roles y privilegios de usuarios TLM sincronizados con Google Cloud IAM (us-east1) y Cloud Run por Juan Yaya.</v>
+        <v>Retención calculada en Cloud SQL: $152.130 COP.</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>mod-1792008371042-27</v>
+        <v>mod-sql-gguz9tq</v>
       </c>
       <c r="B4" t="str">
-        <v>2026-10-14T20:06:11.042Z</v>
+        <v>2026-10-22 14:10:08.991+00</v>
       </c>
       <c r="C4" t="str">
         <v>Juan Yaya</v>
       </c>
-      <c r="D4" t="str">
-        <v>automatizaciones@tlm.net.co</v>
-      </c>
-      <c r="E4" t="str">
-        <v>Administrador</v>
-      </c>
       <c r="F4" t="str">
-        <v>COLABORACION</v>
+        <v>FACTURA_UPDATE</v>
       </c>
       <c r="G4" t="str">
-        <v>Creación de usuario Test Usuario (Analista) con contraseña provisional asignada por Juan</v>
+        <v>Ajuste tributario F350 en SMVP137803: tarifa 2.5%, casilla 64</v>
       </c>
       <c r="H4" t="str">
-        <v>v2-43a1130</v>
+        <v>csql-6vpa8zf</v>
       </c>
       <c r="I4" t="str">
         <v>v2.0</v>
@@ -717,33 +699,27 @@
         <v>Repositorio Central de Juan Yaya</v>
       </c>
       <c r="K4" t="str">
-        <v>Cuenta activada con requisito forzado de cambio de clave al primer ingreso. Notificación enviada a test.user@tlm.net.co.</v>
+        <v>Retención calculada en Cloud SQL: $38.033 COP.</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>mod-1791898676706-988</v>
+        <v>mod-sql-jgg1nhu</v>
       </c>
       <c r="B5" t="str">
-        <v>2026-10-13T13:37:56.706Z</v>
+        <v>2026-10-22 14:10:06.856+00</v>
       </c>
       <c r="C5" t="str">
-        <v>Juan Yaya - Administrador Maestro</v>
-      </c>
-      <c r="D5" t="str">
-        <v>automatizaciones@tlm.net.co</v>
-      </c>
-      <c r="E5" t="str">
-        <v>Administrador</v>
+        <v>Juan Yaya</v>
       </c>
       <c r="F5" t="str">
-        <v>FACTURA_AUDITADA</v>
+        <v>FACTURA_UPDATE</v>
       </c>
       <c r="G5" t="str">
-        <v>Importación automática de factura DRV-3435 desde Google Drive</v>
+        <v>Ajuste tributario F350 en SMVP137803: tarifa 3.5%, casilla 63</v>
       </c>
       <c r="H5" t="str">
-        <v>v2-3b027e4</v>
+        <v>csql-n5t13zw</v>
       </c>
       <c r="I5" t="str">
         <v>v2.0</v>
@@ -752,33 +728,27 @@
         <v>Repositorio Central de Juan Yaya</v>
       </c>
       <c r="K5" t="str">
-        <v>Archivo procesado exitosamente desde la carpeta Google Drive compartida (Consola TLM - Enterprise Repositorio v2.0 (Drive Maestro)).</v>
+        <v>Retención calculada en Cloud SQL: $53.246 COP.</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>mod-1791898672785-307</v>
+        <v>mod-sql-r20gre1</v>
       </c>
       <c r="B6" t="str">
-        <v>2026-10-13T13:37:52.785Z</v>
+        <v>2026-10-22 14:10:03.773+00</v>
       </c>
       <c r="C6" t="str">
-        <v>Juan Yaya - Administrador Maestro</v>
-      </c>
-      <c r="D6" t="str">
-        <v>automatizaciones@tlm.net.co</v>
-      </c>
-      <c r="E6" t="str">
-        <v>Administrador</v>
+        <v>Juan Yaya</v>
       </c>
       <c r="F6" t="str">
-        <v>GCP_SYNC</v>
+        <v>FACTURA_UPDATE</v>
       </c>
       <c r="G6" t="str">
-        <v>Sincronización a Google Drive Corporativo de Juan Yaya (drv-14frw8x)</v>
+        <v>Ajuste tributario F350 en SMVP137803: tarifa 4%, casilla 62</v>
       </c>
       <c r="H6" t="str">
-        <v>v2-375afe4</v>
+        <v>csql-qugqjxq</v>
       </c>
       <c r="I6" t="str">
         <v>v2.0</v>
@@ -787,33 +757,27 @@
         <v>Repositorio Central de Juan Yaya</v>
       </c>
       <c r="K6" t="str">
-        <v>Snapshot y 5 comprobantes DIAN respaldados en carpeta Google Drive (automatizaciones@tlm.net.co).</v>
+        <v>Retención calculada en Cloud SQL: $60.852 COP.</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>mod-1791559570606-221</v>
+        <v>mod-sql-esq6bq5</v>
       </c>
       <c r="B7" t="str">
-        <v>2026-10-09T15:26:10.606Z</v>
+        <v>2026-10-22 12:53:22.135+00</v>
       </c>
       <c r="C7" t="str">
-        <v>Juan David Ramírez</v>
-      </c>
-      <c r="D7" t="str">
-        <v>juan.ramirez@tlm.net.co</v>
-      </c>
-      <c r="E7" t="str">
-        <v>Analista</v>
+        <v>Juan Yaya</v>
       </c>
       <c r="F7" t="str">
-        <v>CONFIG_UPDATE</v>
+        <v>FACTURA_AUDITADA</v>
       </c>
       <c r="G7" t="str">
-        <v>Actualización de contraseña segura alfanumérica para Juan David Ramírez</v>
+        <v>Cambio de estado en factura SMVP137803: → AUDITADA</v>
       </c>
       <c r="H7" t="str">
-        <v>v2-256250a</v>
+        <v>csql-0ti7yeq</v>
       </c>
       <c r="I7" t="str">
         <v>v2.0</v>
@@ -822,33 +786,27 @@
         <v>Repositorio Central de Juan Yaya</v>
       </c>
       <c r="K7" t="str">
-        <v>Estándar de seguridad de 8+ caracteres alfanuméricos aplicado. Estado: Sin contraseña provisional pendiente.</v>
+        <v>Auditoría registrada en vivo en Google Cloud SQL (peak-sunset-511516-q7).</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>mod-1791559570570-543</v>
+        <v>mod-sql-81lgggi</v>
       </c>
       <c r="B8" t="str">
-        <v>2026-10-09T15:26:10.570Z</v>
+        <v>2026-10-22 12:53:20.767+00</v>
       </c>
       <c r="C8" t="str">
-        <v>Juan Yaya - Administrador Maestro</v>
-      </c>
-      <c r="D8" t="str">
-        <v>automatizaciones@tlm.net.co</v>
-      </c>
-      <c r="E8" t="str">
-        <v>Administrador</v>
+        <v>Juan Yaya</v>
       </c>
       <c r="F8" t="str">
-        <v>COLABORACION</v>
+        <v>PUC_UPDATE</v>
       </c>
       <c r="G8" t="str">
-        <v>Creación de usuario Juan David Ramírez (Analista) con contraseña provisional asignada por Juan</v>
+        <v>Reclasificación PUC en SMVP137803: → 513515</v>
       </c>
       <c r="H8" t="str">
-        <v>v2-559e86c</v>
+        <v>csql-ayqagz9</v>
       </c>
       <c r="I8" t="str">
         <v>v2.0</v>
@@ -857,33 +815,27 @@
         <v>Repositorio Central de Juan Yaya</v>
       </c>
       <c r="K8" t="str">
-        <v>Cuenta activada con requisito forzado de cambio de clave al primer ingreso. Notificación enviada a juan.ramirez@tlm.net.co.</v>
+        <v>Tercero: 830001338 (SUMIMAS SAS)</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>mod-1791558074027-772</v>
+        <v>mod-sql-m2nor35</v>
       </c>
       <c r="B9" t="str">
-        <v>2026-10-09T15:01:14.027Z</v>
+        <v>2026-10-22 12:53:04.439+00</v>
       </c>
       <c r="C9" t="str">
         <v>Juan Yaya</v>
       </c>
-      <c r="D9" t="str">
-        <v>automatizaciones@tlm.net.co</v>
-      </c>
-      <c r="E9" t="str">
-        <v>Administrador</v>
-      </c>
       <c r="F9" t="str">
-        <v>GCP_SYNC</v>
+        <v>PUC_UPDATE</v>
       </c>
       <c r="G9" t="str">
-        <v>Sincronización y despliegue del Repositorio v2.0 a Google Cloud Platform (gcp-gwr9pnm)</v>
+        <v>Reclasificación PUC en SMVP137803: → 510506</v>
       </c>
       <c r="H9" t="str">
-        <v>v2-f24899f</v>
+        <v>csql-4bjjubq</v>
       </c>
       <c r="I9" t="str">
         <v>v2.0</v>
@@ -892,159 +844,257 @@
         <v>Repositorio Central de Juan Yaya</v>
       </c>
       <c r="K9" t="str">
-        <v>Snapshot atómico de base de datos y esquemas contables replicado en infraestructura Google Cloud Run.</v>
+        <v>Tercero: 830001338 (SUMIMAS SAS)</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>mod-v2-004</v>
+        <v>mod-sql-m6ehqsp</v>
       </c>
       <c r="B10" t="str">
-        <v>2026-10-08T16:15:00.000Z</v>
+        <v>2026-10-22 12:52:57.781+00</v>
       </c>
       <c r="C10" t="str">
-        <v>Juan Yaya - Administrador Maestro</v>
-      </c>
-      <c r="D10" t="str">
-        <v>automatizaciones@tlm.net.co</v>
-      </c>
-      <c r="E10" t="str">
-        <v>Administrador</v>
+        <v>Juan Yaya</v>
       </c>
       <c r="F10" t="str">
-        <v>RELEASE_V2</v>
+        <v>FACTURA_UPDATE</v>
       </c>
       <c r="G10" t="str">
-        <v>Consolidación oficial de release: Versión 2.0 emitida en Repositorio Central</v>
+        <v>Ajuste tributario F350 en SMVP137803: tarifa 10%, casilla 61</v>
       </c>
       <c r="H10" t="str">
-        <v>v2-8fa3c01</v>
+        <v>csql-w9oyx81</v>
       </c>
       <c r="I10" t="str">
         <v>v2.0</v>
       </c>
       <c r="J10" t="str">
-        <v>Repositorio Maestro de Juan Yaya</v>
+        <v>Repositorio Central de Juan Yaya</v>
       </c>
       <c r="K10" t="str">
-        <v>Fusión de modificaciones de David Morales y Valentina Castro en rama principal master v2.0</v>
+        <v>Retención calculada en Cloud SQL: $152.130 COP.</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>mod-v2-003</v>
+        <v>mod-sql-nr66t7v</v>
       </c>
       <c r="B11" t="str">
-        <v>2026-10-08T15:58:30.000Z</v>
+        <v>2026-10-22 12:52:53.237+00</v>
       </c>
       <c r="C11" t="str">
-        <v>Valentina Castro Rincón (Gestora de Operaciones &amp; UBL)</v>
-      </c>
-      <c r="D11" t="str">
-        <v>valentina.castro@tlm.net.co</v>
-      </c>
-      <c r="E11" t="str">
-        <v>Analista</v>
+        <v>Juan Yaya</v>
       </c>
       <c r="F11" t="str">
-        <v>FACTURA_AUDITADA</v>
+        <v>FACTURA_UPDATE</v>
       </c>
       <c r="G11" t="str">
-        <v>Auditoría UBL de comprobante FE-2045 y verificación de retenciones 4% DIAN</v>
+        <v>Ajuste tributario F350 en SMVP137803: tarifa 2.5%, casilla 64</v>
       </c>
       <c r="H11" t="str">
-        <v>v2-4ce81b2</v>
+        <v>csql-b3bm5xo</v>
       </c>
       <c r="I11" t="str">
         <v>v2.0</v>
       </c>
       <c r="J11" t="str">
-        <v>Repositorio Maestro de Juan Yaya</v>
+        <v>Repositorio Central de Juan Yaya</v>
       </c>
       <c r="K11" t="str">
-        <v>Aprobada para conciliación bancaria y casillas 62/83 del formulario F350</v>
+        <v>Retención calculada en Cloud SQL: $38.033 COP.</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>mod-v2-002</v>
+        <v>mod-sql-ym1txam</v>
       </c>
       <c r="B12" t="str">
-        <v>2026-10-08T15:35:10.000Z</v>
+        <v>2026-10-22 12:52:49.877+00</v>
       </c>
       <c r="C12" t="str">
-        <v>Andrés Felipe Morales (Especialista Tributario)</v>
-      </c>
-      <c r="D12" t="str">
-        <v>andres.morales@tlm.net.co</v>
-      </c>
-      <c r="E12" t="str">
-        <v>Contador</v>
+        <v>Juan Yaya</v>
       </c>
       <c r="F12" t="str">
-        <v>CONCILIACION</v>
+        <v>FACTURA_UPDATE</v>
       </c>
       <c r="G12" t="str">
-        <v>Cruce automático de extracto Bancolombia con tolerancia de 0.00 COP</v>
+        <v>Ajuste tributario F350 en SMVP137803: tarifa 3.5%, casilla 63</v>
       </c>
       <c r="H12" t="str">
-        <v>v2-1df95e4</v>
+        <v>csql-pse3r2t</v>
       </c>
       <c r="I12" t="str">
         <v>v2.0</v>
       </c>
       <c r="J12" t="str">
-        <v>Repositorio Maestro de Juan Yaya</v>
+        <v>Repositorio Central de Juan Yaya</v>
       </c>
       <c r="K12" t="str">
-        <v>Emparejadas 3 partidas mayores y generado comprobante de ajuste Siigo</v>
+        <v>Retención calculada en Cloud SQL: $53.246 COP.</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>mod-v2-001</v>
+        <v>mod-sql-du2keo3</v>
       </c>
       <c r="B13" t="str">
-        <v>2026-10-08T14:40:00.000Z</v>
+        <v>2026-10-22 12:52:44.882+00</v>
       </c>
       <c r="C13" t="str">
-        <v>Andrés Felipe Morales (Especialista Tributario)</v>
-      </c>
-      <c r="D13" t="str">
-        <v>andres.morales@tlm.net.co</v>
-      </c>
-      <c r="E13" t="str">
-        <v>Contador</v>
+        <v>Juan Yaya</v>
       </c>
       <c r="F13" t="str">
-        <v>PUC_UPDATE</v>
+        <v>FACTURA_UPDATE</v>
       </c>
       <c r="G13" t="str">
-        <v>Actualización de mapeo de retenciones en cuentas 236525 y 236801</v>
+        <v>Ajuste tributario F350 en SMVP137803: tarifa 10%, casilla 61</v>
       </c>
       <c r="H13" t="str">
-        <v>v2-9ab22c7</v>
+        <v>csql-8aun46h</v>
       </c>
       <c r="I13" t="str">
         <v>v2.0</v>
       </c>
       <c r="J13" t="str">
-        <v>Repositorio Maestro de Juan Yaya</v>
+        <v>Repositorio Central de Juan Yaya</v>
       </c>
       <c r="K13" t="str">
-        <v>Sincronizado con centros de costo de TLM Consulting y régimen común</v>
+        <v>Retención calculada en Cloud SQL: $152.130 COP.</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>mod-sql-53gzvgn</v>
+      </c>
+      <c r="B14" t="str">
+        <v>2026-10-21 21:03:08.227+00</v>
+      </c>
+      <c r="C14" t="str">
+        <v>Carlos Mendoza (desarrollo)</v>
+      </c>
+      <c r="F14" t="str">
+        <v>COLABORACION</v>
+      </c>
+      <c r="G14" t="str">
+        <v>Creación de usuario jhon castillo (Auditor) sincronizado con Cloud SQL por Juan</v>
+      </c>
+      <c r="H14" t="str">
+        <v>csql-4gk3lg5</v>
+      </c>
+      <c r="I14" t="str">
+        <v>v2.0</v>
+      </c>
+      <c r="J14" t="str">
+        <v>Repositorio Central de Juan Yaya</v>
+      </c>
+      <c r="K14" t="str">
+        <v>Cuenta activada en PostgreSQL (peak-sunset-511516-q7) con requisito forzado de cambio de clave. Notificación enviada a jhonalexander@tlmnet.com.</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>mod-sql-cqdv42e</v>
+      </c>
+      <c r="B15" t="str">
+        <v>2026-10-21 15:08:05.741+00</v>
+      </c>
+      <c r="C15" t="str">
+        <v>Juan Yaya - Administrador Maestro</v>
+      </c>
+      <c r="F15" t="str">
+        <v>COLABORACION</v>
+      </c>
+      <c r="G15" t="str">
+        <v>Creación de usuario Usuario Verificacion E2E (Contador) sincronizado con Cloud SQL por Juan</v>
+      </c>
+      <c r="H15" t="str">
+        <v>csql-6st0j01</v>
+      </c>
+      <c r="I15" t="str">
+        <v>v2.0</v>
+      </c>
+      <c r="J15" t="str">
+        <v>Repositorio Central de Juan Yaya</v>
+      </c>
+      <c r="K15" t="str">
+        <v>Cuenta activada en PostgreSQL (peak-sunset-511516-q7) con requisito forzado de cambio de clave. Notificación enviada a e2e.test.1792595285642@tlm.net.co.</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <v>mod-sql-ot4xj55</v>
+      </c>
+      <c r="B16" t="str">
+        <v>2026-10-21 15:03:18.458+00</v>
+      </c>
+      <c r="C16" t="str">
+        <v>Juan Yaya - Administrador Maestro</v>
+      </c>
+      <c r="F16" t="str">
+        <v>COLABORACION</v>
+      </c>
+      <c r="G16" t="str">
+        <v>Creación de usuario Test Nuevo User 4 (Analista) sincronizado con Cloud SQL por Juan</v>
+      </c>
+      <c r="H16" t="str">
+        <v>csql-1k6g2j5</v>
+      </c>
+      <c r="I16" t="str">
+        <v>v2.0</v>
+      </c>
+      <c r="J16" t="str">
+        <v>Repositorio Central de Juan Yaya</v>
+      </c>
+      <c r="K16" t="str">
+        <v>Cuenta activada en PostgreSQL (peak-sunset-511516-q7) con requisito forzado de cambio de clave. Notificación enviada a test4.nuevo@tlm.net.co.</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="str">
+        <v>mod-neon-init-01</v>
+      </c>
+      <c r="B17" t="str">
+        <v>2026-10-20 12:08:02.658877+00</v>
+      </c>
+      <c r="C17" t="str">
+        <v>Juan Yaya (Administrador Maestro)</v>
+      </c>
+      <c r="D17" t="str">
+        <v>automatizaciones@tlm.net.co</v>
+      </c>
+      <c r="E17" t="str">
+        <v>Administrador</v>
+      </c>
+      <c r="F17" t="str">
+        <v>CONFIGURACION_BASE_DATOS</v>
+      </c>
+      <c r="G17" t="str">
+        <v>Conexión y despliegue inicial en Neon Serverless PostgreSQL (ep-rough-term-b4jl3vvr)</v>
+      </c>
+      <c r="H17" t="str">
+        <v>csql-neon-001</v>
+      </c>
+      <c r="I17" t="str">
+        <v>v2.0</v>
+      </c>
+      <c r="J17" t="str">
+        <v>Repositorio Central de Juan Yaya</v>
+      </c>
+      <c r="K17" t="str">
+        <v>{"ssl": true, "motor": "Neon Serverless PostgreSQL", "region": "us-east-2"}</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:K13"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:K17"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:U7"/>
+  <dimension ref="A1:U9"/>
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
     <col min="2" max="2" width="18.83203125" customWidth="1"/>
@@ -1136,43 +1186,43 @@
     </row>
     <row r="2">
       <c r="A2">
-        <v>1791898676706</v>
+        <v>102</v>
       </c>
       <c r="B2" t="str">
-        <v>DRV-3435</v>
+        <v>SMVP137803</v>
       </c>
       <c r="C2" t="str">
-        <v>Factura Electrónica de Venta</v>
+        <v>Factura Electrónica</v>
       </c>
       <c r="D2" t="str">
-        <v>2026-10-13</v>
+        <v>2026-10-19</v>
       </c>
       <c r="E2" t="str">
-        <v/>
+        <v>2026-11-18</v>
       </c>
       <c r="F2" t="str">
-        <v>900987654</v>
+        <v>830001338</v>
       </c>
       <c r="G2" t="str">
-        <v>GOOGLE CLOUD &amp; WORKSPACE IRELAND LTD</v>
+        <v>SUMIMAS SAS</v>
       </c>
       <c r="H2" t="str">
-        <v>Suscripción Enterprise Google Workspace Drive + Cloud Storage (30 Usuarios)</v>
+        <v>CANON FIJO - EQUIPOS EN RED</v>
       </c>
       <c r="I2">
         <v>1</v>
       </c>
       <c r="J2">
-        <v>1450000</v>
+        <v>1521302</v>
       </c>
       <c r="K2">
-        <v>1450000</v>
+        <v>1521302</v>
       </c>
       <c r="L2">
-        <v>275500</v>
+        <v>289047</v>
       </c>
       <c r="M2">
-        <v>58000</v>
+        <v>60852</v>
       </c>
       <c r="N2" t="str">
         <v>4%</v>
@@ -1181,63 +1231,63 @@
         <v>62</v>
       </c>
       <c r="P2">
-        <v>1667500</v>
+        <v>1810349</v>
       </c>
       <c r="Q2" t="str">
-        <v>Crédito 30 días</v>
+        <v>Contado</v>
       </c>
       <c r="R2" t="str">
-        <v>Transferencia Electrónica</v>
+        <v>Transferencia Débito</v>
       </c>
       <c r="S2" t="str">
-        <v>51353501 - Servicios de Tecnología &amp; Nube</v>
+        <v>513515</v>
       </c>
       <c r="T2" t="str">
         <v>AUDITADA</v>
       </c>
       <c r="U2" t="str">
-        <v>cufe-drv-5a8af0a2ec8f9</v>
+        <v>76205e529505e1b3639cc15fbf1ece195755015a8f1ed3bdc489ad3de411f85f6d913192561f5aa1e92cda04657aa368</v>
       </c>
     </row>
     <row r="3">
       <c r="A3">
-        <v>1</v>
+        <v>101</v>
       </c>
       <c r="B3" t="str">
-        <v>FE-2045</v>
+        <v>SETT-5667</v>
       </c>
       <c r="C3" t="str">
         <v>COMPRAS</v>
       </c>
       <c r="D3" t="str">
-        <v>2026-03-02</v>
+        <v>2026-10-21</v>
       </c>
       <c r="E3" t="str">
-        <v>2026-04-02</v>
+        <v/>
       </c>
       <c r="F3" t="str">
-        <v>901344550</v>
+        <v>860069921</v>
       </c>
       <c r="G3" t="str">
-        <v>AMAZON WEB SERVICES COLOMBIA S.A.S.</v>
+        <v>MICROSOFT COLOMBIA S.A.S.</v>
       </c>
       <c r="H3" t="str">
-        <v>Servicios de Nube e Infraestructura Cloud Hosting Marzo 2026</v>
+        <v>Licenciamiento Microsoft Azure Enterprise &amp; M365 Business</v>
       </c>
       <c r="I3">
         <v>1</v>
       </c>
       <c r="J3">
-        <v>4850000</v>
+        <v>3950000</v>
       </c>
       <c r="K3">
-        <v>4850000</v>
+        <v>3950000</v>
       </c>
       <c r="L3">
-        <v>921500</v>
+        <v>750500</v>
       </c>
       <c r="M3">
-        <v>194000</v>
+        <v>158000</v>
       </c>
       <c r="N3" t="str">
         <v>4%</v>
@@ -1246,7 +1296,7 @@
         <v>62</v>
       </c>
       <c r="P3">
-        <v>5771500</v>
+        <v>4700500</v>
       </c>
       <c r="Q3" t="str">
         <v>Crédito</v>
@@ -1258,275 +1308,405 @@
         <v>513515</v>
       </c>
       <c r="T3" t="str">
-        <v>AUDITADA</v>
+        <v>PENDIENTE</v>
       </c>
       <c r="U3" t="str">
-        <v>3b08e24483a912bb0e4b8ef9910d93ac76bb1a02931a78cc8283a09a1a2b</v>
+        <v>msft_cufe_8buesxq5upi</v>
       </c>
     </row>
     <row r="4">
       <c r="A4">
-        <v>2</v>
+        <v>32</v>
       </c>
       <c r="B4" t="str">
-        <v>F-9812</v>
+        <v>MTO-502</v>
       </c>
       <c r="C4" t="str">
         <v>COMPRAS</v>
       </c>
       <c r="D4" t="str">
-        <v>2026-03-05</v>
+        <v>2026-03-18</v>
       </c>
       <c r="E4" t="str">
-        <v>2026-03-05</v>
+        <v>2026-03-20</v>
       </c>
       <c r="F4" t="str">
-        <v>860002133</v>
+        <v>900654987</v>
       </c>
       <c r="G4" t="str">
-        <v>PAPELES Y SUMINISTROS DE COLOMBIA LTDA</v>
+        <v>SISTEMAS Y REDES INTEGRALES SAS</v>
       </c>
       <c r="H4" t="str">
-        <v>Resmas de papel bond, tóner para impresoras láser y suministros oficina</v>
+        <v>Mantenimiento preventivo servidores rack y cableado estructurado categoría 6A</v>
       </c>
       <c r="I4">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="J4">
-        <v>145000</v>
+        <v>1250000</v>
       </c>
       <c r="K4">
-        <v>1740000</v>
+        <v>1250000</v>
       </c>
       <c r="L4">
-        <v>330600</v>
+        <v>237500</v>
       </c>
       <c r="M4">
-        <v>43500</v>
+        <v>50000</v>
       </c>
       <c r="N4" t="str">
-        <v>2.5%</v>
+        <v>4%</v>
       </c>
       <c r="O4">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="P4">
-        <v>2070600</v>
+        <v>1487500</v>
       </c>
       <c r="Q4" t="str">
         <v>Contado</v>
       </c>
       <c r="R4" t="str">
-        <v>10 - Efectivo</v>
+        <v>47 - Transferencia Bancaria</v>
       </c>
       <c r="S4" t="str">
-        <v>51953001</v>
+        <v>513505</v>
       </c>
       <c r="T4" t="str">
         <v>PENDIENTE</v>
       </c>
       <c r="U4" t="str">
-        <v>9aa47e11f8b3c41a54db0910f8ca73151b88e10c74ba417bc01fa87629b3</v>
+        <v>22ef871b99a03c5188d0112fa7bca9084129e8401928bcad908127361a9f</v>
       </c>
     </row>
     <row r="5">
       <c r="A5">
-        <v>3</v>
+        <v>31</v>
       </c>
       <c r="B5" t="str">
-        <v>HN-108</v>
+        <v>ARR-045</v>
       </c>
       <c r="C5" t="str">
         <v>COMPRAS</v>
       </c>
       <c r="D5" t="str">
-        <v>2026-03-10</v>
+        <v>2026-03-12</v>
       </c>
       <c r="E5" t="str">
-        <v>2026-03-25</v>
+        <v>2026-03-15</v>
       </c>
       <c r="F5" t="str">
-        <v>900543211</v>
+        <v>890900123</v>
       </c>
       <c r="G5" t="str">
-        <v>DR. GUILLERMO VALENCIA ASESORES TRIBUTARIOS S.A.S.</v>
+        <v>INMOBILIARIA DEL COUNTRY S.A.</v>
       </c>
       <c r="H5" t="str">
-        <v>Asesoría y estructuración en cierre fiscal anual y planeación DIAN 2026</v>
+        <v>Canon de arrendamiento oficina corporativa piso 8 mes de Marzo 2026</v>
       </c>
       <c r="I5">
         <v>1</v>
       </c>
       <c r="J5">
-        <v>6500000</v>
+        <v>5200000</v>
       </c>
       <c r="K5">
-        <v>6500000</v>
+        <v>5200000</v>
       </c>
       <c r="L5">
-        <v>1235000</v>
+        <v>988000</v>
       </c>
       <c r="M5">
-        <v>650000</v>
+        <v>182000</v>
       </c>
       <c r="N5" t="str">
-        <v>10%</v>
+        <v>3.5%</v>
       </c>
       <c r="O5">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="P5">
-        <v>7735000</v>
+        <v>6188000</v>
       </c>
       <c r="Q5" t="str">
-        <v>Crédito</v>
+        <v>Contado</v>
       </c>
       <c r="R5" t="str">
         <v>47 - Transferencia Bancaria</v>
       </c>
       <c r="S5" t="str">
-        <v>511010</v>
+        <v>512010</v>
       </c>
       <c r="T5" t="str">
-        <v>AUDITADA</v>
+        <v>SINCRONIZADA_SIIGO</v>
       </c>
       <c r="U5" t="str">
-        <v>f41a87bc9910d54a2b9187ec0029341ba9e745cc91010db910fa78129cc1</v>
+        <v>11a9f0293cb8401ee78120cc948512dd4a0918efbc77124ba18092cd9910</v>
       </c>
     </row>
     <row r="6">
       <c r="A6">
-        <v>4</v>
+        <v>30</v>
       </c>
       <c r="B6" t="str">
-        <v>ARR-045</v>
+        <v>HN-108</v>
       </c>
       <c r="C6" t="str">
         <v>COMPRAS</v>
       </c>
       <c r="D6" t="str">
-        <v>2026-03-12</v>
+        <v>2026-03-10</v>
       </c>
       <c r="E6" t="str">
-        <v>2026-03-15</v>
+        <v>2026-03-25</v>
       </c>
       <c r="F6" t="str">
-        <v>890900123</v>
+        <v>900543211</v>
       </c>
       <c r="G6" t="str">
-        <v>INMOBILIARIA DEL COUNTRY S.A.</v>
+        <v>DR. GUILLERMO VALENCIA ASESORES TRIBUTARIOS S.A.S.</v>
       </c>
       <c r="H6" t="str">
-        <v>Canon de arrendamiento oficina corporativa piso 8 mes de Marzo 2026</v>
+        <v>Asesoría y estructuración en cierre fiscal anual y planeación DIAN 2026</v>
       </c>
       <c r="I6">
         <v>1</v>
       </c>
       <c r="J6">
-        <v>5200000</v>
+        <v>6500000</v>
       </c>
       <c r="K6">
-        <v>5200000</v>
+        <v>6500000</v>
       </c>
       <c r="L6">
-        <v>988000</v>
+        <v>1235000</v>
       </c>
       <c r="M6">
-        <v>182000</v>
+        <v>650000</v>
       </c>
       <c r="N6" t="str">
-        <v>3.5%</v>
+        <v>10%</v>
       </c>
       <c r="O6">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="P6">
-        <v>6188000</v>
+        <v>7735000</v>
       </c>
       <c r="Q6" t="str">
-        <v>Contado</v>
+        <v>Crédito</v>
       </c>
       <c r="R6" t="str">
         <v>47 - Transferencia Bancaria</v>
       </c>
       <c r="S6" t="str">
-        <v>512010</v>
+        <v>511010</v>
       </c>
       <c r="T6" t="str">
-        <v>SINCRONIZADA_SIIGO</v>
+        <v>AUDITADA</v>
       </c>
       <c r="U6" t="str">
-        <v>11a9f0293cb8401ee78120cc948512dd4a0918efbc77124ba18092cd9910</v>
+        <v>f41a87bc9910d54a2b9187ec0029341ba9e745cc91010db910fa78129cc1</v>
       </c>
     </row>
     <row r="7">
       <c r="A7">
-        <v>5</v>
+        <v>29</v>
       </c>
       <c r="B7" t="str">
-        <v>MTO-502</v>
+        <v>F-9812</v>
       </c>
       <c r="C7" t="str">
         <v>COMPRAS</v>
       </c>
       <c r="D7" t="str">
-        <v>2026-03-18</v>
+        <v>2026-03-05</v>
       </c>
       <c r="E7" t="str">
-        <v>2026-03-20</v>
+        <v>2026-03-05</v>
       </c>
       <c r="F7" t="str">
-        <v>900654987</v>
+        <v>860002133</v>
       </c>
       <c r="G7" t="str">
-        <v>SISTEMAS Y REDES INTEGRALES SAS</v>
+        <v>PAPELES Y SUMINISTROS DE COLOMBIA LTDA</v>
       </c>
       <c r="H7" t="str">
-        <v>Mantenimiento preventivo servidores rack y cableado estructurado categoría 6A</v>
+        <v>Resmas de papel bond, tóner para impresoras láser y suministros oficina</v>
       </c>
       <c r="I7">
-        <v>1</v>
+        <v>12</v>
       </c>
       <c r="J7">
-        <v>1250000</v>
+        <v>145000</v>
       </c>
       <c r="K7">
-        <v>1250000</v>
+        <v>1740000</v>
       </c>
       <c r="L7">
-        <v>237500</v>
+        <v>330600</v>
       </c>
       <c r="M7">
-        <v>50000</v>
+        <v>43500</v>
       </c>
       <c r="N7" t="str">
-        <v>4%</v>
+        <v>2.5%</v>
       </c>
       <c r="O7">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="P7">
-        <v>1487500</v>
+        <v>2070600</v>
       </c>
       <c r="Q7" t="str">
         <v>Contado</v>
       </c>
       <c r="R7" t="str">
-        <v>47 - Transferencia Bancaria</v>
+        <v>10 - Efectivo</v>
       </c>
       <c r="S7" t="str">
-        <v>513505</v>
+        <v>51953001</v>
       </c>
       <c r="T7" t="str">
         <v>PENDIENTE</v>
       </c>
       <c r="U7" t="str">
-        <v>22ef871b99a03c5188d0112fa7bca9084129e8401928bcad908127361a9f</v>
+        <v>9aa47e11f8b3c41a54db0910f8ca73151b88e10c74ba417bc01fa87629b3</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8">
+        <v>28</v>
+      </c>
+      <c r="B8" t="str">
+        <v>FE-2045</v>
+      </c>
+      <c r="C8" t="str">
+        <v>COMPRAS</v>
+      </c>
+      <c r="D8" t="str">
+        <v>2026-03-02</v>
+      </c>
+      <c r="E8" t="str">
+        <v>2026-04-02</v>
+      </c>
+      <c r="F8" t="str">
+        <v>901344550</v>
+      </c>
+      <c r="G8" t="str">
+        <v>AMAZON WEB SERVICES COLOMBIA S.A.S.</v>
+      </c>
+      <c r="H8" t="str">
+        <v>Servicios de Nube e Infraestructura Cloud Hosting Marzo 2026</v>
+      </c>
+      <c r="I8">
+        <v>1</v>
+      </c>
+      <c r="J8">
+        <v>4850000</v>
+      </c>
+      <c r="K8">
+        <v>4850000</v>
+      </c>
+      <c r="L8">
+        <v>921500</v>
+      </c>
+      <c r="M8">
+        <v>194000</v>
+      </c>
+      <c r="N8" t="str">
+        <v>4%</v>
+      </c>
+      <c r="O8">
+        <v>62</v>
+      </c>
+      <c r="P8">
+        <v>5771500</v>
+      </c>
+      <c r="Q8" t="str">
+        <v>Crédito</v>
+      </c>
+      <c r="R8" t="str">
+        <v>47 - Transferencia Bancaria</v>
+      </c>
+      <c r="S8" t="str">
+        <v>513515</v>
+      </c>
+      <c r="T8" t="str">
+        <v>AUDITADA</v>
+      </c>
+      <c r="U8" t="str">
+        <v>3b08e24483a912bb0e4b8ef9910d93ac76bb1a02931a78cc8283a09a1a2b</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9">
+        <v>21</v>
+      </c>
+      <c r="B9" t="str">
+        <v>250832064696</v>
+      </c>
+      <c r="C9" t="str">
+        <v>COMPRAS</v>
+      </c>
+      <c r="D9" t="str">
+        <v>2025-10-08</v>
+      </c>
+      <c r="E9" t="str">
+        <v>2025-10-08</v>
+      </c>
+      <c r="F9" t="str">
+        <v>830001338</v>
+      </c>
+      <c r="G9" t="str">
+        <v>SUMIMAS SAS</v>
+      </c>
+      <c r="H9" t="str">
+        <v>ARR IMPRESORA HP M630 B/N</v>
+      </c>
+      <c r="I9">
+        <v>1</v>
+      </c>
+      <c r="J9">
+        <v>4949679</v>
+      </c>
+      <c r="K9">
+        <v>4949679</v>
+      </c>
+      <c r="L9">
+        <v>940439</v>
+      </c>
+      <c r="M9">
+        <v>123742</v>
+      </c>
+      <c r="N9" t="str">
+        <v>2.5%</v>
+      </c>
+      <c r="O9">
+        <v>64</v>
+      </c>
+      <c r="P9">
+        <v>5890118</v>
+      </c>
+      <c r="Q9" t="str">
+        <v>Crédito</v>
+      </c>
+      <c r="R9" t="str">
+        <v>47 - Transferencia Bancaria</v>
+      </c>
+      <c r="S9" t="str">
+        <v>51953001</v>
+      </c>
+      <c r="T9" t="str">
+        <v>PENDIENTE</v>
+      </c>
+      <c r="U9" t="str">
+        <v>de19ba0bf2f87a2c43d5b7ff1462b8de4574bff599ff5eb76df69ced97eb501f983efd1e1188eb9e3f0e67601b05e552</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:U7"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:U9"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1567,13 +1747,13 @@
         <v>1</v>
       </c>
       <c r="C2" t="str">
-        <v>110505</v>
+        <v>111005</v>
       </c>
       <c r="D2" t="str">
-        <v>Caja General</v>
+        <v>Bancos Nacionales (Moneda Local)</v>
       </c>
       <c r="E2" t="str">
-        <v>DEBITO</v>
+        <v>Débito</v>
       </c>
     </row>
     <row r="3">
@@ -1584,13 +1764,13 @@
         <v>1</v>
       </c>
       <c r="C3" t="str">
-        <v>11100501</v>
+        <v>130505</v>
       </c>
       <c r="D3" t="str">
-        <v>Bancolombia Cta Cte 1023</v>
+        <v>Clientes Nacionales</v>
       </c>
       <c r="E3" t="str">
-        <v>DEBITO</v>
+        <v>Débito</v>
       </c>
     </row>
     <row r="4">
@@ -1601,61 +1781,61 @@
         <v>1</v>
       </c>
       <c r="C4" t="str">
-        <v>11100502</v>
+        <v>220505</v>
       </c>
       <c r="D4" t="str">
-        <v>Banco Davivienda Cta Ahorros 4401</v>
+        <v>Proveedores Nacionales</v>
       </c>
       <c r="E4" t="str">
-        <v>DEBITO</v>
+        <v>Crédito</v>
       </c>
     </row>
     <row r="5">
       <c r="A5">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B5">
         <v>1</v>
       </c>
       <c r="C5" t="str">
-        <v>11100503</v>
+        <v>236525</v>
       </c>
       <c r="D5" t="str">
-        <v>BBVA Colombia Operativa</v>
+        <v>Retención en la Fuente Servicios 4%</v>
       </c>
       <c r="E5" t="str">
-        <v>DEBITO</v>
+        <v>Crédito</v>
       </c>
     </row>
     <row r="6">
       <c r="A6">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B6">
         <v>1</v>
       </c>
       <c r="C6" t="str">
-        <v>13050501</v>
+        <v>236540</v>
       </c>
       <c r="D6" t="str">
-        <v>Clientes Nacionales Comerciales</v>
+        <v>Retención en la Fuente Compras 2.5%</v>
       </c>
       <c r="E6" t="str">
-        <v>DEBITO</v>
+        <v>Crédito</v>
       </c>
     </row>
     <row r="7">
       <c r="A7">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="B7">
         <v>1</v>
       </c>
       <c r="C7" t="str">
-        <v>22050501</v>
+        <v>236540</v>
       </c>
       <c r="D7" t="str">
-        <v>Proveedores Nacionales</v>
+        <v>Retención en la Fuente - Compras (2.5%)</v>
       </c>
       <c r="E7" t="str">
         <v>DEBITO</v>
@@ -1663,16 +1843,16 @@
     </row>
     <row r="8">
       <c r="A8">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="B8">
         <v>1</v>
       </c>
       <c r="C8" t="str">
-        <v>233525</v>
+        <v>236701</v>
       </c>
       <c r="D8" t="str">
-        <v>Honorarios por Pagar</v>
+        <v>Impuesto a las Ventas Retenido (ReteIVA 15%)</v>
       </c>
       <c r="E8" t="str">
         <v>DEBITO</v>
@@ -1680,16 +1860,16 @@
     </row>
     <row r="9">
       <c r="A9">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="B9">
         <v>1</v>
       </c>
       <c r="C9" t="str">
-        <v>233595</v>
+        <v>236801</v>
       </c>
       <c r="D9" t="str">
-        <v>Otros Costos y Gastos por Pagar</v>
+        <v>Impuesto de Industria y Comercio Retenido (ReteICA)</v>
       </c>
       <c r="E9" t="str">
         <v>DEBITO</v>
@@ -1697,50 +1877,50 @@
     </row>
     <row r="10">
       <c r="A10">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="B10">
         <v>1</v>
       </c>
       <c r="C10" t="str">
-        <v>236515</v>
+        <v>240801</v>
       </c>
       <c r="D10" t="str">
-        <v>Retención en la Fuente - Honorarios (10% - 11%)</v>
+        <v>IVA Descontable en Compras 19%</v>
       </c>
       <c r="E10" t="str">
-        <v>DEBITO</v>
+        <v>Débito</v>
       </c>
     </row>
     <row r="11">
       <c r="A11">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="B11">
         <v>1</v>
       </c>
       <c r="C11" t="str">
-        <v>236525</v>
+        <v>240802</v>
       </c>
       <c r="D11" t="str">
-        <v>Retención en la Fuente - Servicios (4%)</v>
+        <v>IVA Generado en Ventas 19%</v>
       </c>
       <c r="E11" t="str">
-        <v>DEBITO</v>
+        <v>Crédito</v>
       </c>
     </row>
     <row r="12">
       <c r="A12">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="B12">
         <v>1</v>
       </c>
       <c r="C12" t="str">
-        <v>236540</v>
+        <v>510506</v>
       </c>
       <c r="D12" t="str">
-        <v>Retención en la Fuente - Compras (2.5%)</v>
+        <v>Sueldos y Salarios Personal</v>
       </c>
       <c r="E12" t="str">
         <v>DEBITO</v>
@@ -1748,33 +1928,33 @@
     </row>
     <row r="13">
       <c r="A13">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="B13">
         <v>1</v>
       </c>
       <c r="C13" t="str">
-        <v>236701</v>
+        <v>511010</v>
       </c>
       <c r="D13" t="str">
-        <v>Impuesto a las Ventas Retenido (ReteIVA 15%)</v>
+        <v>Honorarios Asesoría Jurídica</v>
       </c>
       <c r="E13" t="str">
-        <v>DEBITO</v>
+        <v>Débito</v>
       </c>
     </row>
     <row r="14">
       <c r="A14">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="B14">
         <v>1</v>
       </c>
       <c r="C14" t="str">
-        <v>236801</v>
+        <v>511010</v>
       </c>
       <c r="D14" t="str">
-        <v>Impuesto de Industria y Comercio Retenido (ReteICA)</v>
+        <v>Honorarios Asesoría Tributaria y Legal</v>
       </c>
       <c r="E14" t="str">
         <v>DEBITO</v>
@@ -1782,16 +1962,16 @@
     </row>
     <row r="15">
       <c r="A15">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="B15">
         <v>1</v>
       </c>
       <c r="C15" t="str">
-        <v>510506</v>
+        <v>512010</v>
       </c>
       <c r="D15" t="str">
-        <v>Sueldos y Salarios Personal</v>
+        <v>Arrendamientos Inmuebles Administrativos</v>
       </c>
       <c r="E15" t="str">
         <v>DEBITO</v>
@@ -1799,33 +1979,33 @@
     </row>
     <row r="16">
       <c r="A16">
-        <v>15</v>
+        <v>8</v>
       </c>
       <c r="B16">
         <v>1</v>
       </c>
       <c r="C16" t="str">
-        <v>511010</v>
+        <v>513505</v>
       </c>
       <c r="D16" t="str">
-        <v>Honorarios Asesoría Tributaria y Legal</v>
+        <v>Gastos de Aseo y Vigilancia</v>
       </c>
       <c r="E16" t="str">
-        <v>DEBITO</v>
+        <v>Débito</v>
       </c>
     </row>
     <row r="17">
       <c r="A17">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B17">
         <v>1</v>
       </c>
       <c r="C17" t="str">
-        <v>512010</v>
+        <v>513505</v>
       </c>
       <c r="D17" t="str">
-        <v>Arrendamientos Inmuebles Administrativos</v>
+        <v>Servicios de Mantenimiento y Soporte TI</v>
       </c>
       <c r="E17" t="str">
         <v>DEBITO</v>
@@ -1833,16 +2013,16 @@
     </row>
     <row r="18">
       <c r="A18">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B18">
         <v>1</v>
       </c>
       <c r="C18" t="str">
-        <v>513505</v>
+        <v>513515</v>
       </c>
       <c r="D18" t="str">
-        <v>Servicios de Mantenimiento y Soporte TI</v>
+        <v>Servicios de Telecomunicaciones y Cloud</v>
       </c>
       <c r="E18" t="str">
         <v>DEBITO</v>
@@ -1850,19 +2030,19 @@
     </row>
     <row r="19">
       <c r="A19">
-        <v>18</v>
+        <v>9</v>
       </c>
       <c r="B19">
         <v>1</v>
       </c>
       <c r="C19" t="str">
-        <v>513515</v>
+        <v>513535</v>
       </c>
       <c r="D19" t="str">
-        <v>Servicios de Telecomunicaciones y Cloud</v>
+        <v>Servicios de Computación y Cloud</v>
       </c>
       <c r="E19" t="str">
-        <v>DEBITO</v>
+        <v>Débito</v>
       </c>
     </row>
     <row r="20">
@@ -1891,7 +2071,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J4"/>
+  <dimension ref="A1:J7"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -1945,28 +2125,28 @@
         <v>1</v>
       </c>
       <c r="C2" t="str">
-        <v>22050501</v>
+        <v>220505</v>
       </c>
       <c r="D2" t="str">
         <v>Proveedores Nacionales</v>
       </c>
       <c r="E2" t="str">
-        <v>901344550</v>
+        <v>901234567</v>
       </c>
       <c r="F2" t="str">
-        <v>AMAZON WEB SERVICES COLOMBIA S.A.S.</v>
+        <v>SERVICIOS CLOUD COLOMBIA S.A.S.</v>
       </c>
       <c r="G2">
         <v>0</v>
       </c>
       <c r="H2">
-        <v>5577500</v>
+        <v>0</v>
       </c>
       <c r="I2">
-        <v>5577500</v>
+        <v>5355000</v>
       </c>
       <c r="J2">
-        <v>0</v>
+        <v>5355000</v>
       </c>
     </row>
     <row r="3">
@@ -1977,16 +2157,16 @@
         <v>1</v>
       </c>
       <c r="C3" t="str">
-        <v>22050501</v>
+        <v>220505</v>
       </c>
       <c r="D3" t="str">
         <v>Proveedores Nacionales</v>
       </c>
       <c r="E3" t="str">
-        <v>900543211</v>
+        <v>900876543</v>
       </c>
       <c r="F3" t="str">
-        <v>DR. GUILLERMO VALENCIA ASESORES TRIBUTARIOS S.A.S.</v>
+        <v>CONSULTORÍA JURÍDICA TRIBUTARIA SAS</v>
       </c>
       <c r="G3">
         <v>0</v>
@@ -1995,10 +2175,10 @@
         <v>0</v>
       </c>
       <c r="I3">
-        <v>7085000</v>
+        <v>3808000</v>
       </c>
       <c r="J3">
-        <v>7085000</v>
+        <v>3808000</v>
       </c>
     </row>
     <row r="4">
@@ -2009,33 +2189,129 @@
         <v>1</v>
       </c>
       <c r="C4" t="str">
-        <v>13050501</v>
+        <v>220505</v>
       </c>
       <c r="D4" t="str">
-        <v>Clientes Nacionales</v>
+        <v>Proveedores Nacionales</v>
       </c>
       <c r="E4" t="str">
-        <v>800192345</v>
+        <v>890123456</v>
       </c>
       <c r="F4" t="str">
-        <v>DISTRIBUIDORA AGROINDUSTRIAL DEL VALLE</v>
+        <v>SUMINISTROS Y TECNOLOGÍA ANDINA LTDA</v>
       </c>
       <c r="G4">
-        <v>18500000</v>
+        <v>0</v>
       </c>
       <c r="H4">
-        <v>12000000</v>
+        <v>0</v>
       </c>
       <c r="I4">
-        <v>14200000</v>
+        <v>9282000</v>
       </c>
       <c r="J4">
-        <v>16300000</v>
+        <v>9282000</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5">
+        <v>4</v>
+      </c>
+      <c r="B5">
+        <v>1</v>
+      </c>
+      <c r="C5" t="str">
+        <v>220505</v>
+      </c>
+      <c r="D5" t="str">
+        <v>Proveedores Nacionales</v>
+      </c>
+      <c r="E5" t="str">
+        <v>860987654</v>
+      </c>
+      <c r="F5" t="str">
+        <v>TELECOMUNICACIONES DE OCCIDENTE S.A.</v>
+      </c>
+      <c r="G5">
+        <v>0</v>
+      </c>
+      <c r="H5">
+        <v>0</v>
+      </c>
+      <c r="I5">
+        <v>1428000</v>
+      </c>
+      <c r="J5">
+        <v>1428000</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6">
+        <v>5</v>
+      </c>
+      <c r="B6">
+        <v>1</v>
+      </c>
+      <c r="C6" t="str">
+        <v>220505</v>
+      </c>
+      <c r="D6" t="str">
+        <v>Proveedores Nacionales</v>
+      </c>
+      <c r="E6" t="str">
+        <v>901765432</v>
+      </c>
+      <c r="F6" t="str">
+        <v>PAPELERÍA &amp; DOTACIONES EJECUTIVAS SAS</v>
+      </c>
+      <c r="G6">
+        <v>0</v>
+      </c>
+      <c r="H6">
+        <v>0</v>
+      </c>
+      <c r="I6">
+        <v>1011500</v>
+      </c>
+      <c r="J6">
+        <v>1011500</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7">
+        <v>6</v>
+      </c>
+      <c r="B7">
+        <v>1</v>
+      </c>
+      <c r="C7" t="str">
+        <v>220505</v>
+      </c>
+      <c r="D7" t="str">
+        <v>Proveedores Nacionales</v>
+      </c>
+      <c r="E7" t="str">
+        <v>900112233</v>
+      </c>
+      <c r="F7" t="str">
+        <v>SEGURIDAD INFORMÁTICA Y AUDITORÍA LTDA</v>
+      </c>
+      <c r="G7">
+        <v>0</v>
+      </c>
+      <c r="H7">
+        <v>0</v>
+      </c>
+      <c r="I7">
+        <v>6664000</v>
+      </c>
+      <c r="J7">
+        <v>6664000</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:J4"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:J7"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -2085,52 +2361,52 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="str">
-        <v>BNK-001</v>
+      <c r="A2">
+        <v>6</v>
       </c>
       <c r="B2" t="str">
-        <v>2026-03-02</v>
+        <v>2026-10-15</v>
       </c>
       <c r="C2" t="str">
         <v/>
       </c>
       <c r="D2" t="str">
-        <v>TRANSF AWS CLOUD SERVICIOS FACT 2045</v>
+        <v>Abono Factura Cliente 1024</v>
       </c>
       <c r="E2" t="str">
-        <v>DEBITO</v>
+        <v>INGRESO</v>
       </c>
       <c r="F2">
-        <v>5577500</v>
+        <v>18500000</v>
       </c>
       <c r="G2">
         <v>0</v>
       </c>
       <c r="H2" t="str">
-        <v>SÍ</v>
+        <v>NO</v>
       </c>
       <c r="I2" t="str">
-        <v>LIB-001</v>
+        <v>N/A</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="str">
-        <v>BNK-002</v>
+      <c r="A3">
+        <v>5</v>
       </c>
       <c r="B3" t="str">
-        <v>2026-03-05</v>
+        <v>2026-10-11</v>
       </c>
       <c r="C3" t="str">
         <v/>
       </c>
       <c r="D3" t="str">
-        <v>PAGO SUMINISTROS OFICINA COMPRA F-9812</v>
+        <v>Pago Cheque Papeleria Ejecutiva</v>
       </c>
       <c r="E3" t="str">
-        <v>DEBITO</v>
+        <v>EGRESO</v>
       </c>
       <c r="F3">
-        <v>2027100</v>
+        <v>1011500</v>
       </c>
       <c r="G3">
         <v>0</v>
@@ -2139,27 +2415,27 @@
         <v>SÍ</v>
       </c>
       <c r="I3" t="str">
-        <v>LIB-002</v>
+        <v>N/A</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="str">
-        <v>BNK-003</v>
+      <c r="A4">
+        <v>4</v>
       </c>
       <c r="B4" t="str">
-        <v>2026-03-12</v>
+        <v>2026-10-08</v>
       </c>
       <c r="C4" t="str">
         <v/>
       </c>
       <c r="D4" t="str">
-        <v>TRANSFERENCIA ARRIENDO PISO 8 INMOB COUNTRY</v>
+        <v>Debito Automatico Telecom Occidente</v>
       </c>
       <c r="E4" t="str">
-        <v>DEBITO</v>
+        <v>EGRESO</v>
       </c>
       <c r="F4">
-        <v>6006000</v>
+        <v>1428000</v>
       </c>
       <c r="G4">
         <v>0</v>
@@ -2168,91 +2444,91 @@
         <v>SÍ</v>
       </c>
       <c r="I4" t="str">
-        <v>LIB-004</v>
+        <v>N/A</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="str">
-        <v>BNK-004</v>
+      <c r="A5">
+        <v>3</v>
       </c>
       <c r="B5" t="str">
-        <v>2026-03-15</v>
+        <v>2026-10-06</v>
       </c>
       <c r="C5" t="str">
         <v/>
       </c>
       <c r="D5" t="str">
-        <v>COMISION BANCARIA MANEJO CUENTA PYME</v>
+        <v>Pago Suministros Andina Lote 1</v>
       </c>
       <c r="E5" t="str">
-        <v>DEBITO</v>
+        <v>EGRESO</v>
       </c>
       <c r="F5">
-        <v>45000</v>
+        <v>9282000</v>
       </c>
       <c r="G5">
         <v>0</v>
       </c>
       <c r="H5" t="str">
-        <v>NO</v>
+        <v>SÍ</v>
       </c>
       <c r="I5" t="str">
         <v>N/A</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="str">
-        <v>BNK-005</v>
+      <c r="A6">
+        <v>2</v>
       </c>
       <c r="B6" t="str">
-        <v>2026-03-20</v>
+        <v>2026-10-04</v>
       </c>
       <c r="C6" t="str">
         <v/>
       </c>
       <c r="D6" t="str">
-        <v>GRAVAMEN MOVIMIENTOS FINANCIEROS 4X1000</v>
+        <v>Transferencia Consultoria Juridica</v>
       </c>
       <c r="E6" t="str">
-        <v>DEBITO</v>
+        <v>EGRESO</v>
       </c>
       <c r="F6">
-        <v>54620</v>
+        <v>3808000</v>
       </c>
       <c r="G6">
         <v>0</v>
       </c>
       <c r="H6" t="str">
-        <v>NO</v>
+        <v>SÍ</v>
       </c>
       <c r="I6" t="str">
         <v>N/A</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="str">
-        <v>BNK-006</v>
+      <c r="A7">
+        <v>1</v>
       </c>
       <c r="B7" t="str">
-        <v>2026-03-22</v>
+        <v>2026-10-02</v>
       </c>
       <c r="C7" t="str">
         <v/>
       </c>
       <c r="D7" t="str">
-        <v>TRANSFERENCIA CLIENTE ANDINO ABONO FACT 110</v>
+        <v>Pago Transferencia Serv Cloud Col</v>
       </c>
       <c r="E7" t="str">
-        <v>CREDITO</v>
+        <v>EGRESO</v>
       </c>
       <c r="F7">
-        <v>14200000</v>
+        <v>5355000</v>
       </c>
       <c r="G7">
         <v>0</v>
       </c>
       <c r="H7" t="str">
-        <v>NO</v>
+        <v>SÍ</v>
       </c>
       <c r="I7" t="str">
         <v>N/A</v>
@@ -2310,145 +2586,145 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="str">
-        <v>LIB-001</v>
+      <c r="A2">
+        <v>5</v>
       </c>
       <c r="B2" t="str">
-        <v>2026-03-02</v>
+        <v>2026-10-11</v>
       </c>
       <c r="C2" t="str">
-        <v>Pago Factura FE-2045 AWS Latam</v>
+        <v>Comprobante Egreso CE-405 Papeleria</v>
       </c>
       <c r="D2" t="str">
-        <v>11100502</v>
+        <v>111005</v>
       </c>
       <c r="E2" t="str">
-        <v>901344550</v>
+        <v/>
       </c>
       <c r="F2" t="str">
-        <v>DEBITO</v>
+        <v>EGRESO</v>
       </c>
       <c r="G2">
-        <v>5577500</v>
+        <v>1011500</v>
       </c>
       <c r="H2" t="str">
         <v>SÍ</v>
       </c>
       <c r="I2" t="str">
-        <v>BNK-001</v>
+        <v>N/A</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="str">
-        <v>LIB-002</v>
+      <c r="A3">
+        <v>4</v>
       </c>
       <c r="B3" t="str">
-        <v>2026-03-05</v>
+        <v>2026-10-08</v>
       </c>
       <c r="C3" t="str">
-        <v>Egreso Pago Papeles y Suministros F-9812</v>
+        <v>Comprobante Egreso CE-404 Telecom</v>
       </c>
       <c r="D3" t="str">
-        <v>11100502</v>
+        <v>111005</v>
       </c>
       <c r="E3" t="str">
-        <v>860002133</v>
+        <v/>
       </c>
       <c r="F3" t="str">
-        <v>DEBITO</v>
+        <v>EGRESO</v>
       </c>
       <c r="G3">
-        <v>2027100</v>
+        <v>1428000</v>
       </c>
       <c r="H3" t="str">
         <v>SÍ</v>
       </c>
       <c r="I3" t="str">
-        <v>BNK-002</v>
+        <v>N/A</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="str">
-        <v>LIB-003</v>
+      <c r="A4">
+        <v>3</v>
       </c>
       <c r="B4" t="str">
-        <v>2026-03-10</v>
+        <v>2026-10-06</v>
       </c>
       <c r="C4" t="str">
-        <v>Pago Honorarios Dr. Guillermo Valencia HN-108</v>
+        <v>Comprobante Egreso CE-403 Suministros</v>
       </c>
       <c r="D4" t="str">
-        <v>11100502</v>
+        <v>111005</v>
       </c>
       <c r="E4" t="str">
-        <v>900543211</v>
+        <v/>
       </c>
       <c r="F4" t="str">
-        <v>DEBITO</v>
+        <v>EGRESO</v>
       </c>
       <c r="G4">
-        <v>7085000</v>
+        <v>9282000</v>
       </c>
       <c r="H4" t="str">
-        <v>NO</v>
+        <v>SÍ</v>
       </c>
       <c r="I4" t="str">
         <v>N/A</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="str">
-        <v>LIB-004</v>
+      <c r="A5">
+        <v>2</v>
       </c>
       <c r="B5" t="str">
-        <v>2026-03-12</v>
+        <v>2026-10-04</v>
       </c>
       <c r="C5" t="str">
-        <v>Pago Canon Inmobiliaria Country ARR-045</v>
+        <v>Comprobante Egreso CE-402 Consultoria</v>
       </c>
       <c r="D5" t="str">
-        <v>11100502</v>
+        <v>111005</v>
       </c>
       <c r="E5" t="str">
-        <v>890900123</v>
+        <v/>
       </c>
       <c r="F5" t="str">
-        <v>DEBITO</v>
+        <v>EGRESO</v>
       </c>
       <c r="G5">
-        <v>6006000</v>
+        <v>3808000</v>
       </c>
       <c r="H5" t="str">
         <v>SÍ</v>
       </c>
       <c r="I5" t="str">
-        <v>BNK-003</v>
+        <v>N/A</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="str">
-        <v>LIB-005</v>
+      <c r="A6">
+        <v>1</v>
       </c>
       <c r="B6" t="str">
-        <v>2026-03-18</v>
+        <v>2026-10-02</v>
       </c>
       <c r="C6" t="str">
-        <v>Cheque girado mantenimiento Sistemas y Redes</v>
+        <v>Comprobante Egreso CE-401 Serv Cloud</v>
       </c>
       <c r="D6" t="str">
-        <v>11100502</v>
+        <v>111005</v>
       </c>
       <c r="E6" t="str">
-        <v>900654987</v>
+        <v/>
       </c>
       <c r="F6" t="str">
-        <v>DEBITO</v>
+        <v>EGRESO</v>
       </c>
       <c r="G6">
-        <v>1437500</v>
+        <v>5355000</v>
       </c>
       <c r="H6" t="str">
-        <v>NO</v>
+        <v>SÍ</v>
       </c>
       <c r="I6" t="str">
         <v>N/A</v>
@@ -2522,10 +2798,10 @@
         <v>1</v>
       </c>
       <c r="B2" t="str">
-        <v>Juan Yaya - Administrador Maestro</v>
+        <v>Juan Yaya (Administrador Maestro)</v>
       </c>
       <c r="C2" t="str">
-        <v>automatizaciones@tlm.net.co</v>
+        <v>juan.yaya@tlm.net.co</v>
       </c>
       <c r="D2" t="str">
         <v>Administrador</v>
@@ -2560,13 +2836,13 @@
         <v>2</v>
       </c>
       <c r="B3" t="str">
-        <v>María Paula Gómez (Contadora Senior)</v>
+        <v>Carlos Mendoza (desarrollo)</v>
       </c>
       <c r="C3" t="str">
-        <v>maria.gomez@tlm.net.co</v>
+        <v>automatizaciones@tlm.net.co</v>
       </c>
       <c r="D3" t="str">
-        <v>Contador</v>
+        <v>Administrador</v>
       </c>
       <c r="E3" t="str">
         <v>ACTIVO</v>
@@ -2598,10 +2874,10 @@
         <v>3</v>
       </c>
       <c r="B4" t="str">
-        <v>Carlos Rodríguez (Analista Fiscal)</v>
+        <v>Laura Gómez (Analista Contable)</v>
       </c>
       <c r="C4" t="str">
-        <v>carlos.analista@tlm.net.co</v>
+        <v>laura.gomez@tlm.net.co</v>
       </c>
       <c r="D4" t="str">
         <v>Analista</v>
@@ -2636,10 +2912,10 @@
         <v>4</v>
       </c>
       <c r="B5" t="str">
-        <v>Sofía Herrera (Revisor Fiscal)</v>
+        <v>Diana Torres (Auditora Fiscal)</v>
       </c>
       <c r="C5" t="str">
-        <v>sofia.revisor@externo.co</v>
+        <v>diana.torres@tlm.net.co</v>
       </c>
       <c r="D5" t="str">
         <v>Auditor</v>
@@ -2648,7 +2924,7 @@
         <v>ACTIVO</v>
       </c>
       <c r="F5" t="str">
-        <v>1</v>
+        <v>1, 2</v>
       </c>
       <c r="G5" t="str">
         <v>NO</v>
@@ -2724,7 +3000,7 @@
         <v>ACTIVO</v>
       </c>
       <c r="F7" t="str">
-        <v>1, 2</v>
+        <v>1</v>
       </c>
       <c r="G7" t="str">
         <v>NO</v>
@@ -2736,7 +3012,7 @@
         <v>SÍ</v>
       </c>
       <c r="J7" t="str">
-        <v>SÍ</v>
+        <v>NO</v>
       </c>
       <c r="K7" t="str">
         <v>NO</v>
@@ -2747,16 +3023,16 @@
     </row>
     <row r="8">
       <c r="A8">
-        <v>7</v>
+        <v>21</v>
       </c>
       <c r="B8" t="str">
-        <v>Juan David Ramírez</v>
+        <v>jhon castillo</v>
       </c>
       <c r="C8" t="str">
-        <v>juan.ramirez@tlm.net.co</v>
+        <v>jhonalexander@tlmnet.com</v>
       </c>
       <c r="D8" t="str">
-        <v>Analista</v>
+        <v>Auditor</v>
       </c>
       <c r="E8" t="str">
         <v>ACTIVO</v>
@@ -2771,7 +3047,7 @@
         <v>SÍ</v>
       </c>
       <c r="I8" t="str">
-        <v>SÍ</v>
+        <v>NO</v>
       </c>
       <c r="J8" t="str">
         <v>NO</v>
@@ -3050,7 +3326,7 @@
         <v>https://drive.google.com/drive/folders/1tlm-enterprise-drive-juan-yaya-2026</v>
       </c>
       <c r="I2" t="str">
-        <v>2026-10-13T13:37:52.785Z</v>
+        <v>2026-10-21T15:02:52.666Z</v>
       </c>
     </row>
     <row r="3">
@@ -3079,7 +3355,7 @@
         <v>https://drive.google.com/drive/folders/1tlm-enterprise-drive-juan-yaya-2026</v>
       </c>
       <c r="I3" t="str">
-        <v>2026-10-13T10:37:44.459Z</v>
+        <v>2026-10-21T12:02:52.666Z</v>
       </c>
     </row>
     <row r="4">
@@ -3108,7 +3384,7 @@
         <v>https://drive.google.com/drive/folders/1tlm-enterprise-drive-juan-yaya-2026</v>
       </c>
       <c r="I4" t="str">
-        <v>2026-10-13T05:37:44.459Z</v>
+        <v>2026-10-21T07:02:52.666Z</v>
       </c>
     </row>
     <row r="5">
@@ -3137,7 +3413,7 @@
         <v>https://drive.google.com/drive/folders/1tlm-enterprise-drive-juan-yaya-2026</v>
       </c>
       <c r="I5" t="str">
-        <v>2026-10-12T13:37:44.459Z</v>
+        <v>2026-10-20T15:02:52.666Z</v>
       </c>
     </row>
     <row r="6">
@@ -3166,7 +3442,7 @@
         <v>https://drive.google.com/drive/folders/1tlm-enterprise-drive-juan-yaya-2026</v>
       </c>
       <c r="I6" t="str">
-        <v>2026-10-13T01:37:44.459Z</v>
+        <v>2026-10-21T03:02:52.666Z</v>
       </c>
     </row>
     <row r="7">
@@ -3195,7 +3471,7 @@
         <v>https://drive.google.com/drive/folders/1tlm-enterprise-drive-juan-yaya-2026</v>
       </c>
       <c r="I7" t="str">
-        <v>2026-10-14T19:51:01.962Z</v>
+        <v>2026-10-21T15:02:52.666Z</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Importar useRef en CerebroContableView (la pantalla fallaba al abrirse)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MM9XAV8efiRwWz3NxsfcrZ
</commit_message>
<xml_diff>
--- a/data/tlm_base_de_datos_maestra.xlsx
+++ b/data/tlm_base_de_datos_maestra.xlsx
@@ -433,7 +433,7 @@
         <v>Fecha de Generación</v>
       </c>
       <c r="B3" t="str">
-        <v>22/10/2026, 10:50:53 a. m.</v>
+        <v>26/10/2026, 2:28:53 p. m.</v>
       </c>
     </row>
     <row r="4">
@@ -473,7 +473,7 @@
         <v>Total Facturas DIAN Registradas</v>
       </c>
       <c r="B8">
-        <v>8</v>
+        <v>2</v>
       </c>
     </row>
     <row r="9">
@@ -537,7 +537,7 @@
         <v>Auditorías &amp; Commits Registrados</v>
       </c>
       <c r="B16">
-        <v>16</v>
+        <v>22</v>
       </c>
     </row>
     <row r="17">
@@ -545,7 +545,7 @@
         <v>Valor Total Compras Facturadas (COP)</v>
       </c>
       <c r="B17" t="str">
-        <v>$35.653.567</v>
+        <v>$54.943.229</v>
       </c>
     </row>
     <row r="18">
@@ -565,7 +565,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:K17"/>
+  <dimension ref="A1:K23"/>
   <cols>
     <col min="1" max="1" width="14.83203125" customWidth="1"/>
     <col min="2" max="2" width="24.83203125" customWidth="1"/>
@@ -617,10 +617,10 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>mod-sql-otaz37l</v>
+        <v>mod-sql-4do485g</v>
       </c>
       <c r="B2" t="str">
-        <v>2026-10-22 14:10:11.838+00</v>
+        <v>2026-10-26 02:34:09.416+00</v>
       </c>
       <c r="C2" t="str">
         <v>Juan Yaya</v>
@@ -629,10 +629,10 @@
         <v>FACTURA_UPDATE</v>
       </c>
       <c r="G2" t="str">
-        <v>Ajuste tributario F350 en SMVP137803: tarifa 4%, casilla 62</v>
+        <v>Ajuste tributario F350 en SMVP136507: tarifa 10%, casilla 61</v>
       </c>
       <c r="H2" t="str">
-        <v>csql-2b21t39</v>
+        <v>csql-1pkhvcv</v>
       </c>
       <c r="I2" t="str">
         <v>v2.0</v>
@@ -641,15 +641,15 @@
         <v>Repositorio Central de Juan Yaya</v>
       </c>
       <c r="K2" t="str">
-        <v>Retención calculada en Cloud SQL: $60.852 COP.</v>
+        <v>Retención calculada en Cloud SQL: $56.404 COP.</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>mod-sql-j6np45l</v>
+        <v>mod-sql-l6uvgzt</v>
       </c>
       <c r="B3" t="str">
-        <v>2026-10-22 14:10:10.434+00</v>
+        <v>2026-10-26 02:34:06.274+00</v>
       </c>
       <c r="C3" t="str">
         <v>Juan Yaya</v>
@@ -658,10 +658,10 @@
         <v>FACTURA_UPDATE</v>
       </c>
       <c r="G3" t="str">
-        <v>Ajuste tributario F350 en SMVP137803: tarifa 10%, casilla 61</v>
+        <v>Ajuste tributario F350 en SMVP136507: tarifa 3.5%, casilla 63</v>
       </c>
       <c r="H3" t="str">
-        <v>csql-mrh3o41</v>
+        <v>csql-b3cjj1t</v>
       </c>
       <c r="I3" t="str">
         <v>v2.0</v>
@@ -670,27 +670,27 @@
         <v>Repositorio Central de Juan Yaya</v>
       </c>
       <c r="K3" t="str">
-        <v>Retención calculada en Cloud SQL: $152.130 COP.</v>
+        <v>Retención calculada en Cloud SQL: $19.741 COP.</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>mod-sql-gguz9tq</v>
+        <v>mod-sql-bzzavvn</v>
       </c>
       <c r="B4" t="str">
-        <v>2026-10-22 14:10:08.991+00</v>
+        <v>2026-10-26 02:34:01.613+00</v>
       </c>
       <c r="C4" t="str">
         <v>Juan Yaya</v>
       </c>
       <c r="F4" t="str">
-        <v>FACTURA_UPDATE</v>
+        <v>PUC_UPDATE</v>
       </c>
       <c r="G4" t="str">
-        <v>Ajuste tributario F350 en SMVP137803: tarifa 2.5%, casilla 64</v>
+        <v>Reclasificación PUC en SMVP136507: → 511010</v>
       </c>
       <c r="H4" t="str">
-        <v>csql-6vpa8zf</v>
+        <v>csql-663ikqq</v>
       </c>
       <c r="I4" t="str">
         <v>v2.0</v>
@@ -699,27 +699,27 @@
         <v>Repositorio Central de Juan Yaya</v>
       </c>
       <c r="K4" t="str">
-        <v>Retención calculada en Cloud SQL: $38.033 COP.</v>
+        <v>Tercero: 830001338 (SUMIMAS SAS)</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>mod-sql-jgg1nhu</v>
+        <v>mod-sql-ozk1j31</v>
       </c>
       <c r="B5" t="str">
-        <v>2026-10-22 14:10:06.856+00</v>
+        <v>2026-10-26 02:33:37.446+00</v>
       </c>
       <c r="C5" t="str">
         <v>Juan Yaya</v>
       </c>
       <c r="F5" t="str">
-        <v>FACTURA_UPDATE</v>
+        <v>FACTURA_AUDITADA</v>
       </c>
       <c r="G5" t="str">
-        <v>Ajuste tributario F350 en SMVP137803: tarifa 3.5%, casilla 63</v>
+        <v>Cambio de estado en factura SMVP136507: → AUDITADA</v>
       </c>
       <c r="H5" t="str">
-        <v>csql-n5t13zw</v>
+        <v>csql-ug2ybci</v>
       </c>
       <c r="I5" t="str">
         <v>v2.0</v>
@@ -728,15 +728,15 @@
         <v>Repositorio Central de Juan Yaya</v>
       </c>
       <c r="K5" t="str">
-        <v>Retención calculada en Cloud SQL: $53.246 COP.</v>
+        <v>Auditoría registrada en vivo en Google Cloud SQL (peak-sunset-511516-q7).</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>mod-sql-r20gre1</v>
+        <v>mod-sql-1sl63ek</v>
       </c>
       <c r="B6" t="str">
-        <v>2026-10-22 14:10:03.773+00</v>
+        <v>2026-10-23 19:20:30.67+00</v>
       </c>
       <c r="C6" t="str">
         <v>Juan Yaya</v>
@@ -745,10 +745,10 @@
         <v>FACTURA_UPDATE</v>
       </c>
       <c r="G6" t="str">
-        <v>Ajuste tributario F350 en SMVP137803: tarifa 4%, casilla 62</v>
+        <v>Ajuste tributario F350 en SMVP136507: tarifa 4%, casilla 62</v>
       </c>
       <c r="H6" t="str">
-        <v>csql-qugqjxq</v>
+        <v>csql-j365bq6</v>
       </c>
       <c r="I6" t="str">
         <v>v2.0</v>
@@ -757,27 +757,27 @@
         <v>Repositorio Central de Juan Yaya</v>
       </c>
       <c r="K6" t="str">
-        <v>Retención calculada en Cloud SQL: $60.852 COP.</v>
+        <v>Retención calculada en Cloud SQL: $22.561 COP.</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>mod-sql-esq6bq5</v>
+        <v>mod-sql-pcijfqh</v>
       </c>
       <c r="B7" t="str">
-        <v>2026-10-22 12:53:22.135+00</v>
+        <v>2026-10-22 19:24:40.553+00</v>
       </c>
       <c r="C7" t="str">
         <v>Juan Yaya</v>
       </c>
       <c r="F7" t="str">
-        <v>FACTURA_AUDITADA</v>
+        <v>FACTURA_UPDATE</v>
       </c>
       <c r="G7" t="str">
-        <v>Cambio de estado en factura SMVP137803: → AUDITADA</v>
+        <v>Ajuste tributario F350 en FV20327768: tarifa 4%, casilla 62</v>
       </c>
       <c r="H7" t="str">
-        <v>csql-0ti7yeq</v>
+        <v>csql-vbgrwpk</v>
       </c>
       <c r="I7" t="str">
         <v>v2.0</v>
@@ -786,27 +786,27 @@
         <v>Repositorio Central de Juan Yaya</v>
       </c>
       <c r="K7" t="str">
-        <v>Auditoría registrada en vivo en Google Cloud SQL (peak-sunset-511516-q7).</v>
+        <v>Retención calculada en Cloud SQL: $812 COP.</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>mod-sql-81lgggi</v>
+        <v>mod-sql-otaz37l</v>
       </c>
       <c r="B8" t="str">
-        <v>2026-10-22 12:53:20.767+00</v>
+        <v>2026-10-22 14:10:11.838+00</v>
       </c>
       <c r="C8" t="str">
         <v>Juan Yaya</v>
       </c>
       <c r="F8" t="str">
-        <v>PUC_UPDATE</v>
+        <v>FACTURA_UPDATE</v>
       </c>
       <c r="G8" t="str">
-        <v>Reclasificación PUC en SMVP137803: → 513515</v>
+        <v>Ajuste tributario F350 en SMVP137803: tarifa 4%, casilla 62</v>
       </c>
       <c r="H8" t="str">
-        <v>csql-ayqagz9</v>
+        <v>csql-2b21t39</v>
       </c>
       <c r="I8" t="str">
         <v>v2.0</v>
@@ -815,27 +815,27 @@
         <v>Repositorio Central de Juan Yaya</v>
       </c>
       <c r="K8" t="str">
-        <v>Tercero: 830001338 (SUMIMAS SAS)</v>
+        <v>Retención calculada en Cloud SQL: $60.852 COP.</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>mod-sql-m2nor35</v>
+        <v>mod-sql-j6np45l</v>
       </c>
       <c r="B9" t="str">
-        <v>2026-10-22 12:53:04.439+00</v>
+        <v>2026-10-22 14:10:10.434+00</v>
       </c>
       <c r="C9" t="str">
         <v>Juan Yaya</v>
       </c>
       <c r="F9" t="str">
-        <v>PUC_UPDATE</v>
+        <v>FACTURA_UPDATE</v>
       </c>
       <c r="G9" t="str">
-        <v>Reclasificación PUC en SMVP137803: → 510506</v>
+        <v>Ajuste tributario F350 en SMVP137803: tarifa 10%, casilla 61</v>
       </c>
       <c r="H9" t="str">
-        <v>csql-4bjjubq</v>
+        <v>csql-mrh3o41</v>
       </c>
       <c r="I9" t="str">
         <v>v2.0</v>
@@ -844,15 +844,15 @@
         <v>Repositorio Central de Juan Yaya</v>
       </c>
       <c r="K9" t="str">
-        <v>Tercero: 830001338 (SUMIMAS SAS)</v>
+        <v>Retención calculada en Cloud SQL: $152.130 COP.</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>mod-sql-m6ehqsp</v>
+        <v>mod-sql-gguz9tq</v>
       </c>
       <c r="B10" t="str">
-        <v>2026-10-22 12:52:57.781+00</v>
+        <v>2026-10-22 14:10:08.991+00</v>
       </c>
       <c r="C10" t="str">
         <v>Juan Yaya</v>
@@ -861,10 +861,10 @@
         <v>FACTURA_UPDATE</v>
       </c>
       <c r="G10" t="str">
-        <v>Ajuste tributario F350 en SMVP137803: tarifa 10%, casilla 61</v>
+        <v>Ajuste tributario F350 en SMVP137803: tarifa 2.5%, casilla 64</v>
       </c>
       <c r="H10" t="str">
-        <v>csql-w9oyx81</v>
+        <v>csql-6vpa8zf</v>
       </c>
       <c r="I10" t="str">
         <v>v2.0</v>
@@ -873,15 +873,15 @@
         <v>Repositorio Central de Juan Yaya</v>
       </c>
       <c r="K10" t="str">
-        <v>Retención calculada en Cloud SQL: $152.130 COP.</v>
+        <v>Retención calculada en Cloud SQL: $38.033 COP.</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>mod-sql-nr66t7v</v>
+        <v>mod-sql-jgg1nhu</v>
       </c>
       <c r="B11" t="str">
-        <v>2026-10-22 12:52:53.237+00</v>
+        <v>2026-10-22 14:10:06.856+00</v>
       </c>
       <c r="C11" t="str">
         <v>Juan Yaya</v>
@@ -890,10 +890,10 @@
         <v>FACTURA_UPDATE</v>
       </c>
       <c r="G11" t="str">
-        <v>Ajuste tributario F350 en SMVP137803: tarifa 2.5%, casilla 64</v>
+        <v>Ajuste tributario F350 en SMVP137803: tarifa 3.5%, casilla 63</v>
       </c>
       <c r="H11" t="str">
-        <v>csql-b3bm5xo</v>
+        <v>csql-n5t13zw</v>
       </c>
       <c r="I11" t="str">
         <v>v2.0</v>
@@ -902,15 +902,15 @@
         <v>Repositorio Central de Juan Yaya</v>
       </c>
       <c r="K11" t="str">
-        <v>Retención calculada en Cloud SQL: $38.033 COP.</v>
+        <v>Retención calculada en Cloud SQL: $53.246 COP.</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>mod-sql-ym1txam</v>
+        <v>mod-sql-r20gre1</v>
       </c>
       <c r="B12" t="str">
-        <v>2026-10-22 12:52:49.877+00</v>
+        <v>2026-10-22 14:10:03.773+00</v>
       </c>
       <c r="C12" t="str">
         <v>Juan Yaya</v>
@@ -919,10 +919,10 @@
         <v>FACTURA_UPDATE</v>
       </c>
       <c r="G12" t="str">
-        <v>Ajuste tributario F350 en SMVP137803: tarifa 3.5%, casilla 63</v>
+        <v>Ajuste tributario F350 en SMVP137803: tarifa 4%, casilla 62</v>
       </c>
       <c r="H12" t="str">
-        <v>csql-pse3r2t</v>
+        <v>csql-qugqjxq</v>
       </c>
       <c r="I12" t="str">
         <v>v2.0</v>
@@ -931,27 +931,27 @@
         <v>Repositorio Central de Juan Yaya</v>
       </c>
       <c r="K12" t="str">
-        <v>Retención calculada en Cloud SQL: $53.246 COP.</v>
+        <v>Retención calculada en Cloud SQL: $60.852 COP.</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>mod-sql-du2keo3</v>
+        <v>mod-sql-esq6bq5</v>
       </c>
       <c r="B13" t="str">
-        <v>2026-10-22 12:52:44.882+00</v>
+        <v>2026-10-22 12:53:22.135+00</v>
       </c>
       <c r="C13" t="str">
         <v>Juan Yaya</v>
       </c>
       <c r="F13" t="str">
-        <v>FACTURA_UPDATE</v>
+        <v>FACTURA_AUDITADA</v>
       </c>
       <c r="G13" t="str">
-        <v>Ajuste tributario F350 en SMVP137803: tarifa 10%, casilla 61</v>
+        <v>Cambio de estado en factura SMVP137803: → AUDITADA</v>
       </c>
       <c r="H13" t="str">
-        <v>csql-8aun46h</v>
+        <v>csql-0ti7yeq</v>
       </c>
       <c r="I13" t="str">
         <v>v2.0</v>
@@ -960,27 +960,27 @@
         <v>Repositorio Central de Juan Yaya</v>
       </c>
       <c r="K13" t="str">
-        <v>Retención calculada en Cloud SQL: $152.130 COP.</v>
+        <v>Auditoría registrada en vivo en Google Cloud SQL (peak-sunset-511516-q7).</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>mod-sql-53gzvgn</v>
+        <v>mod-sql-81lgggi</v>
       </c>
       <c r="B14" t="str">
-        <v>2026-10-21 21:03:08.227+00</v>
+        <v>2026-10-22 12:53:20.767+00</v>
       </c>
       <c r="C14" t="str">
-        <v>Carlos Mendoza (desarrollo)</v>
+        <v>Juan Yaya</v>
       </c>
       <c r="F14" t="str">
-        <v>COLABORACION</v>
+        <v>PUC_UPDATE</v>
       </c>
       <c r="G14" t="str">
-        <v>Creación de usuario jhon castillo (Auditor) sincronizado con Cloud SQL por Juan</v>
+        <v>Reclasificación PUC en SMVP137803: → 513515</v>
       </c>
       <c r="H14" t="str">
-        <v>csql-4gk3lg5</v>
+        <v>csql-ayqagz9</v>
       </c>
       <c r="I14" t="str">
         <v>v2.0</v>
@@ -989,27 +989,27 @@
         <v>Repositorio Central de Juan Yaya</v>
       </c>
       <c r="K14" t="str">
-        <v>Cuenta activada en PostgreSQL (peak-sunset-511516-q7) con requisito forzado de cambio de clave. Notificación enviada a jhonalexander@tlmnet.com.</v>
+        <v>Tercero: 830001338 (SUMIMAS SAS)</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>mod-sql-cqdv42e</v>
+        <v>mod-sql-m2nor35</v>
       </c>
       <c r="B15" t="str">
-        <v>2026-10-21 15:08:05.741+00</v>
+        <v>2026-10-22 12:53:04.439+00</v>
       </c>
       <c r="C15" t="str">
-        <v>Juan Yaya - Administrador Maestro</v>
+        <v>Juan Yaya</v>
       </c>
       <c r="F15" t="str">
-        <v>COLABORACION</v>
+        <v>PUC_UPDATE</v>
       </c>
       <c r="G15" t="str">
-        <v>Creación de usuario Usuario Verificacion E2E (Contador) sincronizado con Cloud SQL por Juan</v>
+        <v>Reclasificación PUC en SMVP137803: → 510506</v>
       </c>
       <c r="H15" t="str">
-        <v>csql-6st0j01</v>
+        <v>csql-4bjjubq</v>
       </c>
       <c r="I15" t="str">
         <v>v2.0</v>
@@ -1018,27 +1018,27 @@
         <v>Repositorio Central de Juan Yaya</v>
       </c>
       <c r="K15" t="str">
-        <v>Cuenta activada en PostgreSQL (peak-sunset-511516-q7) con requisito forzado de cambio de clave. Notificación enviada a e2e.test.1792595285642@tlm.net.co.</v>
+        <v>Tercero: 830001338 (SUMIMAS SAS)</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>mod-sql-ot4xj55</v>
+        <v>mod-sql-m6ehqsp</v>
       </c>
       <c r="B16" t="str">
-        <v>2026-10-21 15:03:18.458+00</v>
+        <v>2026-10-22 12:52:57.781+00</v>
       </c>
       <c r="C16" t="str">
-        <v>Juan Yaya - Administrador Maestro</v>
+        <v>Juan Yaya</v>
       </c>
       <c r="F16" t="str">
-        <v>COLABORACION</v>
+        <v>FACTURA_UPDATE</v>
       </c>
       <c r="G16" t="str">
-        <v>Creación de usuario Test Nuevo User 4 (Analista) sincronizado con Cloud SQL por Juan</v>
+        <v>Ajuste tributario F350 en SMVP137803: tarifa 10%, casilla 61</v>
       </c>
       <c r="H16" t="str">
-        <v>csql-1k6g2j5</v>
+        <v>csql-w9oyx81</v>
       </c>
       <c r="I16" t="str">
         <v>v2.0</v>
@@ -1047,33 +1047,27 @@
         <v>Repositorio Central de Juan Yaya</v>
       </c>
       <c r="K16" t="str">
-        <v>Cuenta activada en PostgreSQL (peak-sunset-511516-q7) con requisito forzado de cambio de clave. Notificación enviada a test4.nuevo@tlm.net.co.</v>
+        <v>Retención calculada en Cloud SQL: $152.130 COP.</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>mod-neon-init-01</v>
+        <v>mod-sql-nr66t7v</v>
       </c>
       <c r="B17" t="str">
-        <v>2026-10-20 12:08:02.658877+00</v>
+        <v>2026-10-22 12:52:53.237+00</v>
       </c>
       <c r="C17" t="str">
-        <v>Juan Yaya (Administrador Maestro)</v>
-      </c>
-      <c r="D17" t="str">
-        <v>automatizaciones@tlm.net.co</v>
-      </c>
-      <c r="E17" t="str">
-        <v>Administrador</v>
+        <v>Juan Yaya</v>
       </c>
       <c r="F17" t="str">
-        <v>CONFIGURACION_BASE_DATOS</v>
+        <v>FACTURA_UPDATE</v>
       </c>
       <c r="G17" t="str">
-        <v>Conexión y despliegue inicial en Neon Serverless PostgreSQL (ep-rough-term-b4jl3vvr)</v>
+        <v>Ajuste tributario F350 en SMVP137803: tarifa 2.5%, casilla 64</v>
       </c>
       <c r="H17" t="str">
-        <v>csql-neon-001</v>
+        <v>csql-b3bm5xo</v>
       </c>
       <c r="I17" t="str">
         <v>v2.0</v>
@@ -1082,19 +1076,199 @@
         <v>Repositorio Central de Juan Yaya</v>
       </c>
       <c r="K17" t="str">
+        <v>Retención calculada en Cloud SQL: $38.033 COP.</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="str">
+        <v>mod-sql-ym1txam</v>
+      </c>
+      <c r="B18" t="str">
+        <v>2026-10-22 12:52:49.877+00</v>
+      </c>
+      <c r="C18" t="str">
+        <v>Juan Yaya</v>
+      </c>
+      <c r="F18" t="str">
+        <v>FACTURA_UPDATE</v>
+      </c>
+      <c r="G18" t="str">
+        <v>Ajuste tributario F350 en SMVP137803: tarifa 3.5%, casilla 63</v>
+      </c>
+      <c r="H18" t="str">
+        <v>csql-pse3r2t</v>
+      </c>
+      <c r="I18" t="str">
+        <v>v2.0</v>
+      </c>
+      <c r="J18" t="str">
+        <v>Repositorio Central de Juan Yaya</v>
+      </c>
+      <c r="K18" t="str">
+        <v>Retención calculada en Cloud SQL: $53.246 COP.</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="str">
+        <v>mod-sql-du2keo3</v>
+      </c>
+      <c r="B19" t="str">
+        <v>2026-10-22 12:52:44.882+00</v>
+      </c>
+      <c r="C19" t="str">
+        <v>Juan Yaya</v>
+      </c>
+      <c r="F19" t="str">
+        <v>FACTURA_UPDATE</v>
+      </c>
+      <c r="G19" t="str">
+        <v>Ajuste tributario F350 en SMVP137803: tarifa 10%, casilla 61</v>
+      </c>
+      <c r="H19" t="str">
+        <v>csql-8aun46h</v>
+      </c>
+      <c r="I19" t="str">
+        <v>v2.0</v>
+      </c>
+      <c r="J19" t="str">
+        <v>Repositorio Central de Juan Yaya</v>
+      </c>
+      <c r="K19" t="str">
+        <v>Retención calculada en Cloud SQL: $152.130 COP.</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="str">
+        <v>mod-sql-53gzvgn</v>
+      </c>
+      <c r="B20" t="str">
+        <v>2026-10-21 21:03:08.227+00</v>
+      </c>
+      <c r="C20" t="str">
+        <v>Carlos Mendoza (desarrollo)</v>
+      </c>
+      <c r="F20" t="str">
+        <v>COLABORACION</v>
+      </c>
+      <c r="G20" t="str">
+        <v>Creación de usuario jhon castillo (Auditor) sincronizado con Cloud SQL por Juan</v>
+      </c>
+      <c r="H20" t="str">
+        <v>csql-4gk3lg5</v>
+      </c>
+      <c r="I20" t="str">
+        <v>v2.0</v>
+      </c>
+      <c r="J20" t="str">
+        <v>Repositorio Central de Juan Yaya</v>
+      </c>
+      <c r="K20" t="str">
+        <v>Cuenta activada en PostgreSQL (peak-sunset-511516-q7) con requisito forzado de cambio de clave. Notificación enviada a jhonalexander@tlmnet.com.</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="str">
+        <v>mod-sql-cqdv42e</v>
+      </c>
+      <c r="B21" t="str">
+        <v>2026-10-21 15:08:05.741+00</v>
+      </c>
+      <c r="C21" t="str">
+        <v>Juan Yaya - Administrador Maestro</v>
+      </c>
+      <c r="F21" t="str">
+        <v>COLABORACION</v>
+      </c>
+      <c r="G21" t="str">
+        <v>Creación de usuario Usuario Verificacion E2E (Contador) sincronizado con Cloud SQL por Juan</v>
+      </c>
+      <c r="H21" t="str">
+        <v>csql-6st0j01</v>
+      </c>
+      <c r="I21" t="str">
+        <v>v2.0</v>
+      </c>
+      <c r="J21" t="str">
+        <v>Repositorio Central de Juan Yaya</v>
+      </c>
+      <c r="K21" t="str">
+        <v>Cuenta activada en PostgreSQL (peak-sunset-511516-q7) con requisito forzado de cambio de clave. Notificación enviada a e2e.test.1792595285642@tlm.net.co.</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="str">
+        <v>mod-sql-ot4xj55</v>
+      </c>
+      <c r="B22" t="str">
+        <v>2026-10-21 15:03:18.458+00</v>
+      </c>
+      <c r="C22" t="str">
+        <v>Juan Yaya - Administrador Maestro</v>
+      </c>
+      <c r="F22" t="str">
+        <v>COLABORACION</v>
+      </c>
+      <c r="G22" t="str">
+        <v>Creación de usuario Test Nuevo User 4 (Analista) sincronizado con Cloud SQL por Juan</v>
+      </c>
+      <c r="H22" t="str">
+        <v>csql-1k6g2j5</v>
+      </c>
+      <c r="I22" t="str">
+        <v>v2.0</v>
+      </c>
+      <c r="J22" t="str">
+        <v>Repositorio Central de Juan Yaya</v>
+      </c>
+      <c r="K22" t="str">
+        <v>Cuenta activada en PostgreSQL (peak-sunset-511516-q7) con requisito forzado de cambio de clave. Notificación enviada a test4.nuevo@tlm.net.co.</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="str">
+        <v>mod-neon-init-01</v>
+      </c>
+      <c r="B23" t="str">
+        <v>2026-10-20 12:08:02.658877+00</v>
+      </c>
+      <c r="C23" t="str">
+        <v>Juan Yaya (Administrador Maestro)</v>
+      </c>
+      <c r="D23" t="str">
+        <v>automatizaciones@tlm.net.co</v>
+      </c>
+      <c r="E23" t="str">
+        <v>Administrador</v>
+      </c>
+      <c r="F23" t="str">
+        <v>CONFIGURACION_BASE_DATOS</v>
+      </c>
+      <c r="G23" t="str">
+        <v>Conexión y despliegue inicial en Neon Serverless PostgreSQL (ep-rough-term-b4jl3vvr)</v>
+      </c>
+      <c r="H23" t="str">
+        <v>csql-neon-001</v>
+      </c>
+      <c r="I23" t="str">
+        <v>v2.0</v>
+      </c>
+      <c r="J23" t="str">
+        <v>Repositorio Central de Juan Yaya</v>
+      </c>
+      <c r="K23" t="str">
         <v>{"ssl": true, "motor": "Neon Serverless PostgreSQL", "region": "us-east-2"}</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:K17"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:K23"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:U9"/>
+  <dimension ref="A1:U3"/>
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
     <col min="2" max="2" width="18.83203125" customWidth="1"/>
@@ -1186,19 +1360,19 @@
     </row>
     <row r="2">
       <c r="A2">
-        <v>102</v>
+        <v>105</v>
       </c>
       <c r="B2" t="str">
-        <v>SMVP137803</v>
+        <v>SMVP136506</v>
       </c>
       <c r="C2" t="str">
         <v>Factura Electrónica</v>
       </c>
       <c r="D2" t="str">
-        <v>2026-10-19</v>
+        <v>2026-09-08</v>
       </c>
       <c r="E2" t="str">
-        <v>2026-11-18</v>
+        <v>2026-11-07</v>
       </c>
       <c r="F2" t="str">
         <v>830001338</v>
@@ -1207,31 +1381,31 @@
         <v>SUMIMAS SAS</v>
       </c>
       <c r="H2" t="str">
-        <v>CANON FIJO - EQUIPOS EN RED</v>
+        <v>RENTA/ALQUILER DE EQUIPOS</v>
       </c>
       <c r="I2">
         <v>1</v>
       </c>
       <c r="J2">
-        <v>1521302</v>
+        <v>18286460</v>
       </c>
       <c r="K2">
-        <v>1521302</v>
+        <v>18286460</v>
       </c>
       <c r="L2">
-        <v>289047</v>
+        <v>3474427</v>
       </c>
       <c r="M2">
-        <v>60852</v>
+        <v>457162</v>
       </c>
       <c r="N2" t="str">
-        <v>4%</v>
+        <v>2.5%</v>
       </c>
       <c r="O2">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="P2">
-        <v>1810349</v>
+        <v>21760887</v>
       </c>
       <c r="Q2" t="str">
         <v>Contado</v>
@@ -1240,473 +1414,83 @@
         <v>Transferencia Débito</v>
       </c>
       <c r="S2" t="str">
-        <v>513515</v>
+        <v>519530</v>
       </c>
       <c r="T2" t="str">
-        <v>AUDITADA</v>
+        <v>PENDIENTE</v>
       </c>
       <c r="U2" t="str">
-        <v>76205e529505e1b3639cc15fbf1ece195755015a8f1ed3bdc489ad3de411f85f6d913192561f5aa1e92cda04657aa368</v>
+        <v>84b9e52ba2d1be61b19daeaa6645052108b6994c0f6898e902704d1c1cda9888c0f01856488079c77101d256d7924ddf</v>
       </c>
     </row>
     <row r="3">
       <c r="A3">
-        <v>101</v>
+        <v>104</v>
       </c>
       <c r="B3" t="str">
-        <v>SETT-5667</v>
+        <v>SMVP136476</v>
       </c>
       <c r="C3" t="str">
-        <v>COMPRAS</v>
+        <v>Factura Electrónica</v>
       </c>
       <c r="D3" t="str">
-        <v>2026-10-21</v>
+        <v>2026-09-07</v>
       </c>
       <c r="E3" t="str">
-        <v/>
+        <v>2026-11-06</v>
       </c>
       <c r="F3" t="str">
-        <v>860069921</v>
+        <v>830001338</v>
       </c>
       <c r="G3" t="str">
-        <v>MICROSOFT COLOMBIA S.A.S.</v>
+        <v>SUMIMAS SAS</v>
       </c>
       <c r="H3" t="str">
-        <v>Licenciamiento Microsoft Azure Enterprise &amp; M365 Business</v>
+        <v>RENTA/ALQUILER DE EQUIPOS</v>
       </c>
       <c r="I3">
         <v>1</v>
       </c>
       <c r="J3">
-        <v>3950000</v>
+        <v>27884321</v>
       </c>
       <c r="K3">
-        <v>3950000</v>
+        <v>27884321</v>
       </c>
       <c r="L3">
-        <v>750500</v>
+        <v>5298021</v>
       </c>
       <c r="M3">
-        <v>158000</v>
+        <v>697108</v>
       </c>
       <c r="N3" t="str">
-        <v>4%</v>
+        <v>2.5%</v>
       </c>
       <c r="O3">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="P3">
-        <v>4700500</v>
+        <v>33182342</v>
       </c>
       <c r="Q3" t="str">
-        <v>Crédito</v>
+        <v>Contado</v>
       </c>
       <c r="R3" t="str">
-        <v>47 - Transferencia Bancaria</v>
+        <v>Transferencia Débito</v>
       </c>
       <c r="S3" t="str">
-        <v>513515</v>
+        <v>519530</v>
       </c>
       <c r="T3" t="str">
         <v>PENDIENTE</v>
       </c>
       <c r="U3" t="str">
-        <v>msft_cufe_8buesxq5upi</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4">
-        <v>32</v>
-      </c>
-      <c r="B4" t="str">
-        <v>MTO-502</v>
-      </c>
-      <c r="C4" t="str">
-        <v>COMPRAS</v>
-      </c>
-      <c r="D4" t="str">
-        <v>2026-03-18</v>
-      </c>
-      <c r="E4" t="str">
-        <v>2026-03-20</v>
-      </c>
-      <c r="F4" t="str">
-        <v>900654987</v>
-      </c>
-      <c r="G4" t="str">
-        <v>SISTEMAS Y REDES INTEGRALES SAS</v>
-      </c>
-      <c r="H4" t="str">
-        <v>Mantenimiento preventivo servidores rack y cableado estructurado categoría 6A</v>
-      </c>
-      <c r="I4">
-        <v>1</v>
-      </c>
-      <c r="J4">
-        <v>1250000</v>
-      </c>
-      <c r="K4">
-        <v>1250000</v>
-      </c>
-      <c r="L4">
-        <v>237500</v>
-      </c>
-      <c r="M4">
-        <v>50000</v>
-      </c>
-      <c r="N4" t="str">
-        <v>4%</v>
-      </c>
-      <c r="O4">
-        <v>62</v>
-      </c>
-      <c r="P4">
-        <v>1487500</v>
-      </c>
-      <c r="Q4" t="str">
-        <v>Contado</v>
-      </c>
-      <c r="R4" t="str">
-        <v>47 - Transferencia Bancaria</v>
-      </c>
-      <c r="S4" t="str">
-        <v>513505</v>
-      </c>
-      <c r="T4" t="str">
-        <v>PENDIENTE</v>
-      </c>
-      <c r="U4" t="str">
-        <v>22ef871b99a03c5188d0112fa7bca9084129e8401928bcad908127361a9f</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5">
-        <v>31</v>
-      </c>
-      <c r="B5" t="str">
-        <v>ARR-045</v>
-      </c>
-      <c r="C5" t="str">
-        <v>COMPRAS</v>
-      </c>
-      <c r="D5" t="str">
-        <v>2026-03-12</v>
-      </c>
-      <c r="E5" t="str">
-        <v>2026-03-15</v>
-      </c>
-      <c r="F5" t="str">
-        <v>890900123</v>
-      </c>
-      <c r="G5" t="str">
-        <v>INMOBILIARIA DEL COUNTRY S.A.</v>
-      </c>
-      <c r="H5" t="str">
-        <v>Canon de arrendamiento oficina corporativa piso 8 mes de Marzo 2026</v>
-      </c>
-      <c r="I5">
-        <v>1</v>
-      </c>
-      <c r="J5">
-        <v>5200000</v>
-      </c>
-      <c r="K5">
-        <v>5200000</v>
-      </c>
-      <c r="L5">
-        <v>988000</v>
-      </c>
-      <c r="M5">
-        <v>182000</v>
-      </c>
-      <c r="N5" t="str">
-        <v>3.5%</v>
-      </c>
-      <c r="O5">
-        <v>63</v>
-      </c>
-      <c r="P5">
-        <v>6188000</v>
-      </c>
-      <c r="Q5" t="str">
-        <v>Contado</v>
-      </c>
-      <c r="R5" t="str">
-        <v>47 - Transferencia Bancaria</v>
-      </c>
-      <c r="S5" t="str">
-        <v>512010</v>
-      </c>
-      <c r="T5" t="str">
-        <v>SINCRONIZADA_SIIGO</v>
-      </c>
-      <c r="U5" t="str">
-        <v>11a9f0293cb8401ee78120cc948512dd4a0918efbc77124ba18092cd9910</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6">
-        <v>30</v>
-      </c>
-      <c r="B6" t="str">
-        <v>HN-108</v>
-      </c>
-      <c r="C6" t="str">
-        <v>COMPRAS</v>
-      </c>
-      <c r="D6" t="str">
-        <v>2026-03-10</v>
-      </c>
-      <c r="E6" t="str">
-        <v>2026-03-25</v>
-      </c>
-      <c r="F6" t="str">
-        <v>900543211</v>
-      </c>
-      <c r="G6" t="str">
-        <v>DR. GUILLERMO VALENCIA ASESORES TRIBUTARIOS S.A.S.</v>
-      </c>
-      <c r="H6" t="str">
-        <v>Asesoría y estructuración en cierre fiscal anual y planeación DIAN 2026</v>
-      </c>
-      <c r="I6">
-        <v>1</v>
-      </c>
-      <c r="J6">
-        <v>6500000</v>
-      </c>
-      <c r="K6">
-        <v>6500000</v>
-      </c>
-      <c r="L6">
-        <v>1235000</v>
-      </c>
-      <c r="M6">
-        <v>650000</v>
-      </c>
-      <c r="N6" t="str">
-        <v>10%</v>
-      </c>
-      <c r="O6">
-        <v>61</v>
-      </c>
-      <c r="P6">
-        <v>7735000</v>
-      </c>
-      <c r="Q6" t="str">
-        <v>Crédito</v>
-      </c>
-      <c r="R6" t="str">
-        <v>47 - Transferencia Bancaria</v>
-      </c>
-      <c r="S6" t="str">
-        <v>511010</v>
-      </c>
-      <c r="T6" t="str">
-        <v>AUDITADA</v>
-      </c>
-      <c r="U6" t="str">
-        <v>f41a87bc9910d54a2b9187ec0029341ba9e745cc91010db910fa78129cc1</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7">
-        <v>29</v>
-      </c>
-      <c r="B7" t="str">
-        <v>F-9812</v>
-      </c>
-      <c r="C7" t="str">
-        <v>COMPRAS</v>
-      </c>
-      <c r="D7" t="str">
-        <v>2026-03-05</v>
-      </c>
-      <c r="E7" t="str">
-        <v>2026-03-05</v>
-      </c>
-      <c r="F7" t="str">
-        <v>860002133</v>
-      </c>
-      <c r="G7" t="str">
-        <v>PAPELES Y SUMINISTROS DE COLOMBIA LTDA</v>
-      </c>
-      <c r="H7" t="str">
-        <v>Resmas de papel bond, tóner para impresoras láser y suministros oficina</v>
-      </c>
-      <c r="I7">
-        <v>12</v>
-      </c>
-      <c r="J7">
-        <v>145000</v>
-      </c>
-      <c r="K7">
-        <v>1740000</v>
-      </c>
-      <c r="L7">
-        <v>330600</v>
-      </c>
-      <c r="M7">
-        <v>43500</v>
-      </c>
-      <c r="N7" t="str">
-        <v>2.5%</v>
-      </c>
-      <c r="O7">
-        <v>64</v>
-      </c>
-      <c r="P7">
-        <v>2070600</v>
-      </c>
-      <c r="Q7" t="str">
-        <v>Contado</v>
-      </c>
-      <c r="R7" t="str">
-        <v>10 - Efectivo</v>
-      </c>
-      <c r="S7" t="str">
-        <v>51953001</v>
-      </c>
-      <c r="T7" t="str">
-        <v>PENDIENTE</v>
-      </c>
-      <c r="U7" t="str">
-        <v>9aa47e11f8b3c41a54db0910f8ca73151b88e10c74ba417bc01fa87629b3</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8">
-        <v>28</v>
-      </c>
-      <c r="B8" t="str">
-        <v>FE-2045</v>
-      </c>
-      <c r="C8" t="str">
-        <v>COMPRAS</v>
-      </c>
-      <c r="D8" t="str">
-        <v>2026-03-02</v>
-      </c>
-      <c r="E8" t="str">
-        <v>2026-04-02</v>
-      </c>
-      <c r="F8" t="str">
-        <v>901344550</v>
-      </c>
-      <c r="G8" t="str">
-        <v>AMAZON WEB SERVICES COLOMBIA S.A.S.</v>
-      </c>
-      <c r="H8" t="str">
-        <v>Servicios de Nube e Infraestructura Cloud Hosting Marzo 2026</v>
-      </c>
-      <c r="I8">
-        <v>1</v>
-      </c>
-      <c r="J8">
-        <v>4850000</v>
-      </c>
-      <c r="K8">
-        <v>4850000</v>
-      </c>
-      <c r="L8">
-        <v>921500</v>
-      </c>
-      <c r="M8">
-        <v>194000</v>
-      </c>
-      <c r="N8" t="str">
-        <v>4%</v>
-      </c>
-      <c r="O8">
-        <v>62</v>
-      </c>
-      <c r="P8">
-        <v>5771500</v>
-      </c>
-      <c r="Q8" t="str">
-        <v>Crédito</v>
-      </c>
-      <c r="R8" t="str">
-        <v>47 - Transferencia Bancaria</v>
-      </c>
-      <c r="S8" t="str">
-        <v>513515</v>
-      </c>
-      <c r="T8" t="str">
-        <v>AUDITADA</v>
-      </c>
-      <c r="U8" t="str">
-        <v>3b08e24483a912bb0e4b8ef9910d93ac76bb1a02931a78cc8283a09a1a2b</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9">
-        <v>21</v>
-      </c>
-      <c r="B9" t="str">
-        <v>250832064696</v>
-      </c>
-      <c r="C9" t="str">
-        <v>COMPRAS</v>
-      </c>
-      <c r="D9" t="str">
-        <v>2025-10-08</v>
-      </c>
-      <c r="E9" t="str">
-        <v>2025-10-08</v>
-      </c>
-      <c r="F9" t="str">
-        <v>830001338</v>
-      </c>
-      <c r="G9" t="str">
-        <v>SUMIMAS SAS</v>
-      </c>
-      <c r="H9" t="str">
-        <v>ARR IMPRESORA HP M630 B/N</v>
-      </c>
-      <c r="I9">
-        <v>1</v>
-      </c>
-      <c r="J9">
-        <v>4949679</v>
-      </c>
-      <c r="K9">
-        <v>4949679</v>
-      </c>
-      <c r="L9">
-        <v>940439</v>
-      </c>
-      <c r="M9">
-        <v>123742</v>
-      </c>
-      <c r="N9" t="str">
-        <v>2.5%</v>
-      </c>
-      <c r="O9">
-        <v>64</v>
-      </c>
-      <c r="P9">
-        <v>5890118</v>
-      </c>
-      <c r="Q9" t="str">
-        <v>Crédito</v>
-      </c>
-      <c r="R9" t="str">
-        <v>47 - Transferencia Bancaria</v>
-      </c>
-      <c r="S9" t="str">
-        <v>51953001</v>
-      </c>
-      <c r="T9" t="str">
-        <v>PENDIENTE</v>
-      </c>
-      <c r="U9" t="str">
-        <v>de19ba0bf2f87a2c43d5b7ff1462b8de4574bff599ff5eb76df69ced97eb501f983efd1e1188eb9e3f0e67601b05e552</v>
+        <v>98b2548002b2cfb7f853768525eb340949638bafbb75cf9942befbef4f529b8702667951001e4e868ed1141678d6329d</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:U9"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:U3"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -2739,7 +2523,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L8"/>
+  <dimension ref="A1:N8"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="28.83203125" customWidth="1"/>
@@ -2753,6 +2537,8 @@
     <col min="10" max="10" width="20.83203125" customWidth="1"/>
     <col min="11" max="11" width="16.83203125" customWidth="1"/>
     <col min="12" max="12" width="16.83203125" customWidth="1"/>
+    <col min="13" max="13" width="16.83203125" customWidth="1"/>
+    <col min="14" max="14" width="16.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2792,6 +2578,12 @@
       <c r="L1" t="str">
         <v>GESTION USUARIOS</v>
       </c>
+      <c r="M1" t="str">
+        <v>BASE DE DATOS</v>
+      </c>
+      <c r="N1" t="str">
+        <v>ARQUITECTURA ESCALA</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2">
@@ -2829,6 +2621,12 @@
       </c>
       <c r="L2" t="str">
         <v>SÍ</v>
+      </c>
+      <c r="M2" t="str">
+        <v>NO</v>
+      </c>
+      <c r="N2" t="str">
+        <v>NO</v>
       </c>
     </row>
     <row r="3">
@@ -2868,6 +2666,12 @@
       <c r="L3" t="str">
         <v>NO</v>
       </c>
+      <c r="M3" t="str">
+        <v>NO</v>
+      </c>
+      <c r="N3" t="str">
+        <v>NO</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4">
@@ -2898,12 +2702,18 @@
         <v>SÍ</v>
       </c>
       <c r="J4" t="str">
-        <v>NO</v>
+        <v>SÍ</v>
       </c>
       <c r="K4" t="str">
         <v>NO</v>
       </c>
       <c r="L4" t="str">
+        <v>NO</v>
+      </c>
+      <c r="M4" t="str">
+        <v>NO</v>
+      </c>
+      <c r="N4" t="str">
         <v>NO</v>
       </c>
     </row>
@@ -2944,6 +2754,12 @@
       <c r="L5" t="str">
         <v>NO</v>
       </c>
+      <c r="M5" t="str">
+        <v>NO</v>
+      </c>
+      <c r="N5" t="str">
+        <v>NO</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6">
@@ -2982,6 +2798,12 @@
       <c r="L6" t="str">
         <v>NO</v>
       </c>
+      <c r="M6" t="str">
+        <v>NO</v>
+      </c>
+      <c r="N6" t="str">
+        <v>NO</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7">
@@ -3020,6 +2842,12 @@
       <c r="L7" t="str">
         <v>NO</v>
       </c>
+      <c r="M7" t="str">
+        <v>NO</v>
+      </c>
+      <c r="N7" t="str">
+        <v>NO</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8">
@@ -3058,10 +2886,16 @@
       <c r="L8" t="str">
         <v>NO</v>
       </c>
+      <c r="M8" t="str">
+        <v>NO</v>
+      </c>
+      <c r="N8" t="str">
+        <v>NO</v>
+      </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:L8"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:N8"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>